<commit_message>
Fix paper table and smoke-test reporting
</commit_message>
<xml_diff>
--- a/paper/data/shareable/manuscript_tables/DELPHI_Supplementary_Table_5.xlsx
+++ b/paper/data/shareable/manuscript_tables/DELPHI_Supplementary_Table_5.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jain2017" sheetId="1" r:id="R344b0930e2e54158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDPa1" sheetId="2" r:id="Rfe8a8105da804431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDPa3" sheetId="3" r:id="R149683c2571047e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jain2017" sheetId="1" r:id="R68809ee5d34640c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDPa1" sheetId="2" r:id="Rda0ac4b42f4b417a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDPa3" sheetId="3" r:id="R67cb16395ace4e99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.000000"/>
+  </x:numFmts>
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -26,13 +29,24 @@
       <x:sz val="11"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="2">
@@ -55,7 +69,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -64,6 +78,15 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -13926,57 +13949,64 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8.83203125" style="3" customWidth="0"/>
+    <x:col min="1" max="1" width="14" style="3" hidden="0" customWidth="1"/>
     <x:col min="2" max="3" width="46.33203125" style="3" customWidth="1"/>
     <x:col min="4" max="8" width="8.83203125" style="3" customWidth="0"/>
     <x:col min="9" max="14" width="20.6640625" style="3" customWidth="1"/>
     <x:col min="15" max="15" width="20.6640625" style="2" customWidth="1"/>
     <x:col min="16" max="16384" width="8.83203125" style="2" customWidth="0"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="64">
-      <x:c r="A1" s="1" t="str">
+      <x:c r="A1" s="5" t="str">
         <x:v>antibody_id</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>HSEQ</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>LSEQ</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>CDR3</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>polyreactivity_prscore_cho_avg</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="str">
-        <x:v>psr_filter_cho</x:v>
-      </x:c>
-      <x:c r="G1" s="1" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>polyreactivity_prscore_ova_avg</x:v>
       </x:c>
-      <x:c r="H1" s="1" t="str">
-        <x:v>psr_filter_ova</x:v>
-      </x:c>
-      <x:c r="I1" s="1" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>transformer_lm_ablang_ipi_psr_trainset_score</x:v>
       </x:c>
-      <x:c r="J1" s="1" t="str">
+      <x:c r="H1" s="5" t="str">
         <x:v>transformer_lm_antiberty_ipi_psr_trainset_score</x:v>
       </x:c>
-      <x:c r="K1" s="1" t="str">
+      <x:c r="I1" s="5" t="str">
         <x:v>transformer_lm_antiberta2_ipi_psr_trainset_score</x:v>
       </x:c>
-      <x:c r="L1" s="1" t="str">
+      <x:c r="J1" s="5" t="str">
         <x:v>transformer_lm_antiberta2-cssp_ipi_psr_trainset_score</x:v>
       </x:c>
-      <x:c r="M1" s="1" t="str">
+      <x:c r="K1" s="5" t="str">
         <x:v>transformer_lm_igbert_ipi_psr_trainset_score</x:v>
       </x:c>
-      <x:c r="N1" s="1" t="str">
+      <x:c r="L1" s="5" t="str">
         <x:v>transformer_onehot_onehot_ipi_psr_trainset_score</x:v>
       </x:c>
+      <x:c r="M1" s="1"/>
+      <x:c r="N1" s="1"/>
     </x:row>
     <x:row r="2" ht="48">
       <x:c r="A2" s="3" t="str">
@@ -13991,36 +14021,32 @@
       <x:c r="D2" s="3" t="str">
         <x:v>TLGDY</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="n">
+      <x:c r="E2" s="6" t="n">
         <x:v>0.0456680817627101</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G2" s="3" t="n">
+      <x:c r="F2" s="6" t="n">
         <x:v>0.02362932236366475</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I2" s="3" t="n">
+      <x:c r="G2" s="6" t="n">
         <x:v>0.9680544137954712</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="n">
+      <x:c r="H2" s="6" t="n">
         <x:v>0.9958482980728149</x:v>
       </x:c>
-      <x:c r="K2" s="3" t="n">
+      <x:c r="I2" s="6" t="n">
         <x:v>0.9964450001716614</x:v>
       </x:c>
-      <x:c r="L2" s="3" t="n">
+      <x:c r="J2" s="6" t="n">
         <x:v>0.9182215929031372</x:v>
       </x:c>
-      <x:c r="M2" s="3" t="n">
+      <x:c r="K2" s="6" t="n">
         <x:v>0.9806955456733704</x:v>
       </x:c>
-      <x:c r="N2" s="3" t="n">
+      <x:c r="L2" s="6" t="n">
         <x:v>0.9944287538528442</x:v>
       </x:c>
+      <x:c r="M2" s="3"/>
+      <x:c r="N2" s="3"/>
     </x:row>
     <x:row r="3" ht="48">
       <x:c r="A3" s="3" t="str">
@@ -14035,36 +14061,32 @@
       <x:c r="D3" s="3" t="str">
         <x:v>MIFGA</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="n">
+      <x:c r="E3" s="6" t="n">
         <x:v>0.1071337289612092</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G3" s="3" t="n">
+      <x:c r="F3" s="6" t="n">
         <x:v>0.111900766792193</x:v>
       </x:c>
-      <x:c r="H3" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I3" s="3" t="n">
+      <x:c r="G3" s="6" t="n">
         <x:v>0.7701752185821533</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="n">
+      <x:c r="H3" s="6" t="n">
         <x:v>0.9741355180740356</x:v>
       </x:c>
-      <x:c r="K3" s="3" t="n">
+      <x:c r="I3" s="6" t="n">
         <x:v>0.9673761129379272</x:v>
       </x:c>
-      <x:c r="L3" s="3" t="n">
+      <x:c r="J3" s="6" t="n">
         <x:v>0.875627875328064</x:v>
       </x:c>
-      <x:c r="M3" s="3" t="n">
+      <x:c r="K3" s="6" t="n">
         <x:v>0.1732734739780426</x:v>
       </x:c>
-      <x:c r="N3" s="3" t="n">
+      <x:c r="L3" s="6" t="n">
         <x:v>0.7458527684211731</x:v>
       </x:c>
+      <x:c r="M3" s="3"/>
+      <x:c r="N3" s="3"/>
     </x:row>
     <x:row r="4" ht="48">
       <x:c r="A4" s="3" t="str">
@@ -14079,36 +14101,32 @@
       <x:c r="D4" s="3" t="str">
         <x:v>TPGDY</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="n">
+      <x:c r="E4" s="6" t="n">
         <x:v>0.3636807335734132</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G4" s="3" t="n">
+      <x:c r="F4" s="6" t="n">
         <x:v>0.06882350645691646</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I4" s="3" t="n">
+      <x:c r="G4" s="6" t="n">
         <x:v>0.5081616640090942</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="n">
+      <x:c r="H4" s="6" t="n">
         <x:v>0.9976351261138916</x:v>
       </x:c>
-      <x:c r="K4" s="3" t="n">
+      <x:c r="I4" s="6" t="n">
         <x:v>0.9975074529647827</x:v>
       </x:c>
-      <x:c r="L4" s="3" t="n">
+      <x:c r="J4" s="6" t="n">
         <x:v>0.9145091772079468</x:v>
       </x:c>
-      <x:c r="M4" s="3" t="n">
+      <x:c r="K4" s="6" t="n">
         <x:v>0.979477047920227</x:v>
       </x:c>
-      <x:c r="N4" s="3" t="n">
+      <x:c r="L4" s="6" t="n">
         <x:v>0.9945323467254639</x:v>
       </x:c>
+      <x:c r="M4" s="3"/>
+      <x:c r="N4" s="3"/>
     </x:row>
     <x:row r="5" ht="48">
       <x:c r="A5" s="3" t="str">
@@ -14123,36 +14141,32 @@
       <x:c r="D5" s="3" t="str">
         <x:v>AITYF</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G5" s="3" t="n">
+      <x:c r="E5" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="n">
         <x:v>0.07778538764313558</x:v>
       </x:c>
-      <x:c r="H5" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I5" s="3" t="n">
+      <x:c r="G5" s="6" t="n">
         <x:v>0.00234873010776937</x:v>
       </x:c>
-      <x:c r="J5" s="3" t="n">
+      <x:c r="H5" s="6" t="n">
         <x:v>0.9710049629211426</x:v>
       </x:c>
-      <x:c r="K5" s="3" t="n">
+      <x:c r="I5" s="6" t="n">
         <x:v>0.3625645339488983</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="n">
+      <x:c r="J5" s="6" t="n">
         <x:v>0.3098916709423065</x:v>
       </x:c>
-      <x:c r="M5" s="3" t="n">
+      <x:c r="K5" s="6" t="n">
         <x:v>0.8693008422851562</x:v>
       </x:c>
-      <x:c r="N5" s="3" t="n">
+      <x:c r="L5" s="6" t="n">
         <x:v>0.2285288721323013</x:v>
       </x:c>
+      <x:c r="M5" s="3"/>
+      <x:c r="N5" s="3"/>
     </x:row>
     <x:row r="6" ht="48">
       <x:c r="A6" s="3" t="str">
@@ -14167,36 +14181,32 @@
       <x:c r="D6" s="3" t="str">
         <x:v>MTGGGY</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="n">
+      <x:c r="E6" s="6" t="n">
         <x:v>0.1040975157241797</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="n">
+      <x:c r="F6" s="6" t="n">
         <x:v>0.100244495737974</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I6" s="3" t="n">
+      <x:c r="G6" s="6" t="n">
         <x:v>0.05003084987401962</x:v>
       </x:c>
-      <x:c r="J6" s="3" t="n">
+      <x:c r="H6" s="6" t="n">
         <x:v>0.9882773756980896</x:v>
       </x:c>
-      <x:c r="K6" s="3" t="n">
+      <x:c r="I6" s="6" t="n">
         <x:v>0.9950266480445862</x:v>
       </x:c>
-      <x:c r="L6" s="3" t="n">
+      <x:c r="J6" s="6" t="n">
         <x:v>0.9920565485954285</x:v>
       </x:c>
-      <x:c r="M6" s="3" t="n">
+      <x:c r="K6" s="6" t="n">
         <x:v>0.9649059772491455</x:v>
       </x:c>
-      <x:c r="N6" s="3" t="n">
+      <x:c r="L6" s="6" t="n">
         <x:v>0.9908308982849121</x:v>
       </x:c>
+      <x:c r="M6" s="3"/>
+      <x:c r="N6" s="3"/>
     </x:row>
     <x:row r="7" ht="48">
       <x:c r="A7" s="3" t="str">
@@ -14211,36 +14221,32 @@
       <x:c r="D7" s="3" t="str">
         <x:v>GTPGIP</x:v>
       </x:c>
-      <x:c r="E7" s="3" t="n">
+      <x:c r="E7" s="6" t="n">
         <x:v>0.163142129845978</x:v>
       </x:c>
-      <x:c r="F7" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G7" s="3" t="n">
+      <x:c r="F7" s="6" t="n">
         <x:v>0.102322113300521</x:v>
       </x:c>
-      <x:c r="H7" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I7" s="3" t="n">
+      <x:c r="G7" s="6" t="n">
         <x:v>0.8760566115379333</x:v>
       </x:c>
-      <x:c r="J7" s="3" t="n">
+      <x:c r="H7" s="6" t="n">
         <x:v>0.9939579963684082</x:v>
       </x:c>
-      <x:c r="K7" s="3" t="n">
+      <x:c r="I7" s="6" t="n">
         <x:v>0.9374638199806213</x:v>
       </x:c>
-      <x:c r="L7" s="3" t="n">
+      <x:c r="J7" s="6" t="n">
         <x:v>0.2007558196783066</x:v>
       </x:c>
-      <x:c r="M7" s="3" t="n">
+      <x:c r="K7" s="6" t="n">
         <x:v>0.005308525636792183</x:v>
       </x:c>
-      <x:c r="N7" s="3" t="n">
+      <x:c r="L7" s="6" t="n">
         <x:v>0.984978199005127</x:v>
       </x:c>
+      <x:c r="M7" s="3"/>
+      <x:c r="N7" s="3"/>
     </x:row>
     <x:row r="8" ht="48">
       <x:c r="A8" s="3" t="str">
@@ -14255,36 +14261,32 @@
       <x:c r="D8" s="3" t="str">
         <x:v>ARTSDT</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="n">
+      <x:c r="E8" s="6" t="n">
         <x:v>0.09134852450682505</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="n">
+      <x:c r="F8" s="6" t="n">
         <x:v>0.1009339041332135</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I8" s="3" t="n">
+      <x:c r="G8" s="6" t="n">
         <x:v>0.001676026149652898</x:v>
       </x:c>
-      <x:c r="J8" s="3" t="n">
+      <x:c r="H8" s="6" t="n">
         <x:v>0.001801666687242687</x:v>
       </x:c>
-      <x:c r="K8" s="3" t="n">
+      <x:c r="I8" s="6" t="n">
         <x:v>0.01240196451544762</x:v>
       </x:c>
-      <x:c r="L8" s="3" t="n">
+      <x:c r="J8" s="6" t="n">
         <x:v>0.001591825275681913</x:v>
       </x:c>
-      <x:c r="M8" s="3" t="n">
+      <x:c r="K8" s="6" t="n">
         <x:v>0.001302246702834964</x:v>
       </x:c>
-      <x:c r="N8" s="3" t="n">
+      <x:c r="L8" s="6" t="n">
         <x:v>0.9955524802207947</x:v>
       </x:c>
+      <x:c r="M8" s="3"/>
+      <x:c r="N8" s="3"/>
     </x:row>
     <x:row r="9" ht="48">
       <x:c r="A9" s="3" t="str">
@@ -14299,36 +14301,32 @@
       <x:c r="D9" s="3" t="str">
         <x:v>ASNLVH</x:v>
       </x:c>
-      <x:c r="E9" s="3" t="n">
+      <x:c r="E9" s="6" t="n">
         <x:v>0.006192235830194975</x:v>
       </x:c>
-      <x:c r="F9" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G9" s="3" t="n">
+      <x:c r="F9" s="6" t="n">
         <x:v>0.04257497049357375</x:v>
       </x:c>
-      <x:c r="H9" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I9" s="3" t="n">
+      <x:c r="G9" s="6" t="n">
         <x:v>0.9707611203193665</x:v>
       </x:c>
-      <x:c r="J9" s="3" t="n">
+      <x:c r="H9" s="6" t="n">
         <x:v>0.9939627051353455</x:v>
       </x:c>
-      <x:c r="K9" s="3" t="n">
+      <x:c r="I9" s="6" t="n">
         <x:v>0.9842162728309631</x:v>
       </x:c>
-      <x:c r="L9" s="3" t="n">
+      <x:c r="J9" s="6" t="n">
         <x:v>0.9893691539764404</x:v>
       </x:c>
-      <x:c r="M9" s="3" t="n">
+      <x:c r="K9" s="6" t="n">
         <x:v>0.8094174861907959</x:v>
       </x:c>
-      <x:c r="N9" s="3" t="n">
+      <x:c r="L9" s="6" t="n">
         <x:v>0.5401731133460999</x:v>
       </x:c>
+      <x:c r="M9" s="3"/>
+      <x:c r="N9" s="3"/>
     </x:row>
     <x:row r="10" ht="48">
       <x:c r="A10" s="3" t="str">
@@ -14343,36 +14341,32 @@
       <x:c r="D10" s="3" t="str">
         <x:v>ARQGLDV</x:v>
       </x:c>
-      <x:c r="E10" s="3" t="n">
+      <x:c r="E10" s="6" t="n">
         <x:v>0.10107346764399</x:v>
       </x:c>
-      <x:c r="F10" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G10" s="3" t="n">
+      <x:c r="F10" s="6" t="n">
         <x:v>0.06907170549432858</x:v>
       </x:c>
-      <x:c r="H10" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I10" s="3" t="n">
+      <x:c r="G10" s="6" t="n">
         <x:v>0.02268993109464645</x:v>
       </x:c>
-      <x:c r="J10" s="3" t="n">
+      <x:c r="H10" s="6" t="n">
         <x:v>0.9968692660331726</x:v>
       </x:c>
-      <x:c r="K10" s="3" t="n">
+      <x:c r="I10" s="6" t="n">
         <x:v>0.991051435470581</x:v>
       </x:c>
-      <x:c r="L10" s="3" t="n">
+      <x:c r="J10" s="6" t="n">
         <x:v>0.995546817779541</x:v>
       </x:c>
-      <x:c r="M10" s="3" t="n">
+      <x:c r="K10" s="6" t="n">
         <x:v>0.5286281704902649</x:v>
       </x:c>
-      <x:c r="N10" s="3" t="n">
+      <x:c r="L10" s="6" t="n">
         <x:v>0.9937898516654968</x:v>
       </x:c>
+      <x:c r="M10" s="3"/>
+      <x:c r="N10" s="3"/>
     </x:row>
     <x:row r="11" ht="48">
       <x:c r="A11" s="3" t="str">
@@ -14387,36 +14381,32 @@
       <x:c r="D11" s="3" t="str">
         <x:v>ITKNVPD</x:v>
       </x:c>
-      <x:c r="E11" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G11" s="3" t="n">
+      <x:c r="E11" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="n">
         <x:v>0.1003537476531061</x:v>
       </x:c>
-      <x:c r="H11" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I11" s="3" t="n">
+      <x:c r="G11" s="6" t="n">
         <x:v>0.001632568426430225</x:v>
       </x:c>
-      <x:c r="J11" s="3" t="n">
+      <x:c r="H11" s="6" t="n">
         <x:v>0.995294988155365</x:v>
       </x:c>
-      <x:c r="K11" s="3" t="n">
+      <x:c r="I11" s="6" t="n">
         <x:v>0.9909375905990601</x:v>
       </x:c>
-      <x:c r="L11" s="3" t="n">
+      <x:c r="J11" s="6" t="n">
         <x:v>0.9749261736869812</x:v>
       </x:c>
-      <x:c r="M11" s="3" t="n">
+      <x:c r="K11" s="6" t="n">
         <x:v>0.003858848242089152</x:v>
       </x:c>
-      <x:c r="N11" s="3" t="n">
+      <x:c r="L11" s="6" t="n">
         <x:v>0.9974862337112427</x:v>
       </x:c>
+      <x:c r="M11" s="3"/>
+      <x:c r="N11" s="3"/>
     </x:row>
     <x:row r="12" ht="48">
       <x:c r="A12" s="3" t="str">
@@ -14431,36 +14421,32 @@
       <x:c r="D12" s="3" t="str">
         <x:v>ARDFTDV</x:v>
       </x:c>
-      <x:c r="E12" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="n">
+      <x:c r="E12" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="n">
         <x:v>0.04353999810796737</x:v>
       </x:c>
-      <x:c r="H12" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I12" s="3" t="n">
+      <x:c r="G12" s="6" t="n">
         <x:v>0.9623173475265503</x:v>
       </x:c>
-      <x:c r="J12" s="3" t="n">
+      <x:c r="H12" s="6" t="n">
         <x:v>0.3488620817661285</x:v>
       </x:c>
-      <x:c r="K12" s="3" t="n">
+      <x:c r="I12" s="6" t="n">
         <x:v>0.9267259240150452</x:v>
       </x:c>
-      <x:c r="L12" s="3" t="n">
+      <x:c r="J12" s="6" t="n">
         <x:v>0.2368784993886948</x:v>
       </x:c>
-      <x:c r="M12" s="3" t="n">
+      <x:c r="K12" s="6" t="n">
         <x:v>0.923877477645874</x:v>
       </x:c>
-      <x:c r="N12" s="3" t="n">
+      <x:c r="L12" s="6" t="n">
         <x:v>0.9945422410964966</x:v>
       </x:c>
+      <x:c r="M12" s="3"/>
+      <x:c r="N12" s="3"/>
     </x:row>
     <x:row r="13" ht="48">
       <x:c r="A13" s="3" t="str">
@@ -14475,36 +14461,32 @@
       <x:c r="D13" s="3" t="str">
         <x:v>VKVVTTE</x:v>
       </x:c>
-      <x:c r="E13" s="3" t="n">
+      <x:c r="E13" s="6" t="n">
         <x:v>0.09253663433766772</x:v>
       </x:c>
-      <x:c r="F13" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G13" s="3" t="n">
+      <x:c r="F13" s="6" t="n">
         <x:v>0.14558727800653</x:v>
       </x:c>
-      <x:c r="H13" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I13" s="3" t="n">
+      <x:c r="G13" s="6" t="n">
         <x:v>0.6651975512504578</x:v>
       </x:c>
-      <x:c r="J13" s="3" t="n">
+      <x:c r="H13" s="6" t="n">
         <x:v>0.9915992021560669</x:v>
       </x:c>
-      <x:c r="K13" s="3" t="n">
+      <x:c r="I13" s="6" t="n">
         <x:v>0.9215853214263916</x:v>
       </x:c>
-      <x:c r="L13" s="3" t="n">
+      <x:c r="J13" s="6" t="n">
         <x:v>0.04849838092923164</x:v>
       </x:c>
-      <x:c r="M13" s="3" t="n">
+      <x:c r="K13" s="6" t="n">
         <x:v>0.9940646290779114</x:v>
       </x:c>
-      <x:c r="N13" s="3" t="n">
+      <x:c r="L13" s="6" t="n">
         <x:v>0.9967334270477295</x:v>
       </x:c>
+      <x:c r="M13" s="3"/>
+      <x:c r="N13" s="3"/>
     </x:row>
     <x:row r="14" ht="48">
       <x:c r="A14" s="3" t="str">
@@ -14519,36 +14501,32 @@
       <x:c r="D14" s="3" t="str">
         <x:v>ASNWNFQH</x:v>
       </x:c>
-      <x:c r="E14" s="3" t="n">
+      <x:c r="E14" s="6" t="n">
         <x:v>0.3317476373043587</x:v>
       </x:c>
-      <x:c r="F14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="3" t="n">
+      <x:c r="F14" s="6" t="n">
         <x:v>0.24845998053019</x:v>
       </x:c>
-      <x:c r="H14" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I14" s="3" t="n">
+      <x:c r="G14" s="6" t="n">
         <x:v>0.1523776352405548</x:v>
       </x:c>
-      <x:c r="J14" s="3" t="n">
+      <x:c r="H14" s="6" t="n">
         <x:v>0.001244410523213446</x:v>
       </x:c>
-      <x:c r="K14" s="3" t="n">
+      <x:c r="I14" s="6" t="n">
         <x:v>0.4459444880485535</x:v>
       </x:c>
-      <x:c r="L14" s="3" t="n">
+      <x:c r="J14" s="6" t="n">
         <x:v>0.01173305511474609</x:v>
       </x:c>
-      <x:c r="M14" s="3" t="n">
+      <x:c r="K14" s="6" t="n">
         <x:v>0.9465925693511963</x:v>
       </x:c>
-      <x:c r="N14" s="3" t="n">
+      <x:c r="L14" s="6" t="n">
         <x:v>0.9920530319213867</x:v>
       </x:c>
+      <x:c r="M14" s="3"/>
+      <x:c r="N14" s="3"/>
     </x:row>
     <x:row r="15" ht="48">
       <x:c r="A15" s="3" t="str">
@@ -14563,36 +14541,32 @@
       <x:c r="D15" s="3" t="str">
         <x:v>AKDIPLDS</x:v>
       </x:c>
-      <x:c r="E15" s="3" t="n">
+      <x:c r="E15" s="6" t="n">
         <x:v>0.00935246348388435</x:v>
       </x:c>
-      <x:c r="F15" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G15" s="3" t="n">
+      <x:c r="F15" s="6" t="n">
         <x:v>0.05780373652127973</x:v>
       </x:c>
-      <x:c r="H15" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I15" s="3" t="n">
+      <x:c r="G15" s="6" t="n">
         <x:v>0.7747852206230164</x:v>
       </x:c>
-      <x:c r="J15" s="3" t="n">
+      <x:c r="H15" s="6" t="n">
         <x:v>0.9963642954826355</x:v>
       </x:c>
-      <x:c r="K15" s="3" t="n">
+      <x:c r="I15" s="6" t="n">
         <x:v>0.990160346031189</x:v>
       </x:c>
-      <x:c r="L15" s="3" t="n">
+      <x:c r="J15" s="6" t="n">
         <x:v>0.9579960107803345</x:v>
       </x:c>
-      <x:c r="M15" s="3" t="n">
+      <x:c r="K15" s="6" t="n">
         <x:v>0.9828333854675293</x:v>
       </x:c>
-      <x:c r="N15" s="3" t="n">
+      <x:c r="L15" s="6" t="n">
         <x:v>0.9961724877357483</x:v>
       </x:c>
+      <x:c r="M15" s="3"/>
+      <x:c r="N15" s="3"/>
     </x:row>
     <x:row r="16" ht="48">
       <x:c r="A16" s="3" t="str">
@@ -14607,36 +14581,32 @@
       <x:c r="D16" s="3" t="str">
         <x:v>ARGRDIDF</x:v>
       </x:c>
-      <x:c r="E16" s="3" t="n">
+      <x:c r="E16" s="6" t="n">
         <x:v>0.166511516060456</x:v>
       </x:c>
-      <x:c r="F16" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G16" s="3" t="n">
+      <x:c r="F16" s="6" t="n">
         <x:v>0.06229089464337428</x:v>
       </x:c>
-      <x:c r="H16" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I16" s="3" t="n">
+      <x:c r="G16" s="6" t="n">
         <x:v>0.4031769931316376</x:v>
       </x:c>
-      <x:c r="J16" s="3" t="n">
+      <x:c r="H16" s="6" t="n">
         <x:v>0.9971311092376709</x:v>
       </x:c>
-      <x:c r="K16" s="3" t="n">
+      <x:c r="I16" s="6" t="n">
         <x:v>0.9968589544296265</x:v>
       </x:c>
-      <x:c r="L16" s="3" t="n">
+      <x:c r="J16" s="6" t="n">
         <x:v>0.9902438521385193</x:v>
       </x:c>
-      <x:c r="M16" s="3" t="n">
+      <x:c r="K16" s="6" t="n">
         <x:v>0.9183588027954102</x:v>
       </x:c>
-      <x:c r="N16" s="3" t="n">
+      <x:c r="L16" s="6" t="n">
         <x:v>0.9970704317092896</x:v>
       </x:c>
+      <x:c r="M16" s="3"/>
+      <x:c r="N16" s="3"/>
     </x:row>
     <x:row r="17" ht="48">
       <x:c r="A17" s="3" t="str">
@@ -14651,36 +14621,32 @@
       <x:c r="D17" s="3" t="str">
         <x:v>ARGGYFDY</x:v>
       </x:c>
-      <x:c r="E17" s="3" t="n">
+      <x:c r="E17" s="6" t="n">
         <x:v>0.00122080801661905</x:v>
       </x:c>
-      <x:c r="F17" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G17" s="3" t="n">
+      <x:c r="F17" s="6" t="n">
         <x:v>0.0126001840020047</x:v>
       </x:c>
-      <x:c r="H17" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I17" s="3" t="n">
+      <x:c r="G17" s="6" t="n">
         <x:v>0.4553740620613098</x:v>
       </x:c>
-      <x:c r="J17" s="3" t="n">
+      <x:c r="H17" s="6" t="n">
         <x:v>0.9957063794136047</x:v>
       </x:c>
-      <x:c r="K17" s="3" t="n">
+      <x:c r="I17" s="6" t="n">
         <x:v>0.9833549857139587</x:v>
       </x:c>
-      <x:c r="L17" s="3" t="n">
+      <x:c r="J17" s="6" t="n">
         <x:v>0.9964325428009033</x:v>
       </x:c>
-      <x:c r="M17" s="3" t="n">
+      <x:c r="K17" s="6" t="n">
         <x:v>0.007857115939259529</x:v>
       </x:c>
-      <x:c r="N17" s="3" t="n">
+      <x:c r="L17" s="6" t="n">
         <x:v>0.9940648674964905</x:v>
       </x:c>
+      <x:c r="M17" s="3"/>
+      <x:c r="N17" s="3"/>
     </x:row>
     <x:row r="18" ht="48">
       <x:c r="A18" s="3" t="str">
@@ -14695,36 +14661,32 @@
       <x:c r="D18" s="3" t="str">
         <x:v>ARDRIAIFS</x:v>
       </x:c>
-      <x:c r="E18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F18" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G18" s="3" t="n">
+      <x:c r="E18" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="n">
         <x:v>0.06243850047681965</x:v>
       </x:c>
-      <x:c r="H18" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I18" s="3" t="n">
+      <x:c r="G18" s="6" t="n">
         <x:v>0.5509874224662781</x:v>
       </x:c>
-      <x:c r="J18" s="3" t="n">
+      <x:c r="H18" s="6" t="n">
         <x:v>0.01052233204245567</x:v>
       </x:c>
-      <x:c r="K18" s="3" t="n">
+      <x:c r="I18" s="6" t="n">
         <x:v>0.912674069404602</x:v>
       </x:c>
-      <x:c r="L18" s="3" t="n">
+      <x:c r="J18" s="6" t="n">
         <x:v>0.990978479385376</x:v>
       </x:c>
-      <x:c r="M18" s="3" t="n">
+      <x:c r="K18" s="6" t="n">
         <x:v>0.04800922051072121</x:v>
       </x:c>
-      <x:c r="N18" s="3" t="n">
+      <x:c r="L18" s="6" t="n">
         <x:v>0.9965314269065857</x:v>
       </x:c>
+      <x:c r="M18" s="3"/>
+      <x:c r="N18" s="3"/>
     </x:row>
     <x:row r="19" ht="48">
       <x:c r="A19" s="3" t="str">
@@ -14739,36 +14701,32 @@
       <x:c r="D19" s="3" t="str">
         <x:v>ARSTWYFDS</x:v>
       </x:c>
-      <x:c r="E19" s="3" t="n">
+      <x:c r="E19" s="6" t="n">
         <x:v>0.4598809296994095</x:v>
       </x:c>
-      <x:c r="F19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="3" t="n">
+      <x:c r="F19" s="6" t="n">
         <x:v>0.3908363303664638</x:v>
       </x:c>
-      <x:c r="H19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" s="3" t="n">
+      <x:c r="G19" s="6" t="n">
         <x:v>0.005234695971012115</x:v>
       </x:c>
-      <x:c r="J19" s="3" t="n">
+      <x:c r="H19" s="6" t="n">
         <x:v>0.9762315154075623</x:v>
       </x:c>
-      <x:c r="K19" s="3" t="n">
+      <x:c r="I19" s="6" t="n">
         <x:v>0.9774358868598938</x:v>
       </x:c>
-      <x:c r="L19" s="3" t="n">
+      <x:c r="J19" s="6" t="n">
         <x:v>0.9441280364990234</x:v>
       </x:c>
-      <x:c r="M19" s="3" t="n">
+      <x:c r="K19" s="6" t="n">
         <x:v>0.5804517269134521</x:v>
       </x:c>
-      <x:c r="N19" s="3" t="n">
+      <x:c r="L19" s="6" t="n">
         <x:v>0.995908260345459</x:v>
       </x:c>
+      <x:c r="M19" s="3"/>
+      <x:c r="N19" s="3"/>
     </x:row>
     <x:row r="20" ht="48">
       <x:c r="A20" s="3" t="str">
@@ -14783,36 +14741,32 @@
       <x:c r="D20" s="3" t="str">
         <x:v>ARAYDSLDV</x:v>
       </x:c>
-      <x:c r="E20" s="3" t="n">
+      <x:c r="E20" s="6" t="n">
         <x:v>0.0725356450106452</x:v>
       </x:c>
-      <x:c r="F20" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G20" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H20" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I20" s="3" t="n">
+      <x:c r="F20" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="n">
         <x:v>0.8529093861579895</x:v>
       </x:c>
-      <x:c r="J20" s="3" t="n">
+      <x:c r="H20" s="6" t="n">
         <x:v>0.9941583871841431</x:v>
       </x:c>
-      <x:c r="K20" s="3" t="n">
+      <x:c r="I20" s="6" t="n">
         <x:v>0.9926659464836121</x:v>
       </x:c>
-      <x:c r="L20" s="3" t="n">
+      <x:c r="J20" s="6" t="n">
         <x:v>0.9890641570091248</x:v>
       </x:c>
-      <x:c r="M20" s="3" t="n">
+      <x:c r="K20" s="6" t="n">
         <x:v>0.5850761532783508</x:v>
       </x:c>
-      <x:c r="N20" s="3" t="n">
+      <x:c r="L20" s="6" t="n">
         <x:v>0.9914195537567139</x:v>
       </x:c>
+      <x:c r="M20" s="3"/>
+      <x:c r="N20" s="3"/>
     </x:row>
     <x:row r="21" ht="48">
       <x:c r="A21" s="3" t="str">
@@ -14827,36 +14781,32 @@
       <x:c r="D21" s="3" t="str">
         <x:v>ASSGFYFDF</x:v>
       </x:c>
-      <x:c r="E21" s="3" t="n">
+      <x:c r="E21" s="6" t="n">
         <x:v>0.284071648639038</x:v>
       </x:c>
-      <x:c r="F21" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G21" s="3" t="n">
+      <x:c r="F21" s="6" t="n">
         <x:v>0.1174059523823555</x:v>
       </x:c>
-      <x:c r="H21" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I21" s="3" t="n">
+      <x:c r="G21" s="6" t="n">
         <x:v>0.002242353744804859</x:v>
       </x:c>
-      <x:c r="J21" s="3" t="n">
+      <x:c r="H21" s="6" t="n">
         <x:v>0.9428451061248779</x:v>
       </x:c>
-      <x:c r="K21" s="3" t="n">
+      <x:c r="I21" s="6" t="n">
         <x:v>0.5295020341873169</x:v>
       </x:c>
-      <x:c r="L21" s="3" t="n">
+      <x:c r="J21" s="6" t="n">
         <x:v>0.7935394048690796</x:v>
       </x:c>
-      <x:c r="M21" s="3" t="n">
+      <x:c r="K21" s="6" t="n">
         <x:v>0.7135488390922546</x:v>
       </x:c>
-      <x:c r="N21" s="3" t="n">
+      <x:c r="L21" s="6" t="n">
         <x:v>0.9828681945800781</x:v>
       </x:c>
+      <x:c r="M21" s="3"/>
+      <x:c r="N21" s="3"/>
     </x:row>
     <x:row r="22" ht="48">
       <x:c r="A22" s="3" t="str">
@@ -14871,36 +14821,32 @@
       <x:c r="D22" s="3" t="str">
         <x:v>AKEDWGLPRD</x:v>
       </x:c>
-      <x:c r="E22" s="3" t="n">
+      <x:c r="E22" s="6" t="n">
         <x:v>0.000416134718457725</x:v>
       </x:c>
-      <x:c r="F22" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G22" s="3" t="n">
+      <x:c r="F22" s="6" t="n">
         <x:v>0.03805320147998442</x:v>
       </x:c>
-      <x:c r="H22" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I22" s="3" t="n">
+      <x:c r="G22" s="6" t="n">
         <x:v>0.06958945840597153</x:v>
       </x:c>
-      <x:c r="J22" s="3" t="n">
+      <x:c r="H22" s="6" t="n">
         <x:v>0.9787682890892029</x:v>
       </x:c>
-      <x:c r="K22" s="3" t="n">
+      <x:c r="I22" s="6" t="n">
         <x:v>0.8581089377403259</x:v>
       </x:c>
-      <x:c r="L22" s="3" t="n">
+      <x:c r="J22" s="6" t="n">
         <x:v>0.01151434704661369</x:v>
       </x:c>
-      <x:c r="M22" s="3" t="n">
+      <x:c r="K22" s="6" t="n">
         <x:v>0.7989660501480103</x:v>
       </x:c>
-      <x:c r="N22" s="3" t="n">
+      <x:c r="L22" s="6" t="n">
         <x:v>0.993509829044342</x:v>
       </x:c>
+      <x:c r="M22" s="3"/>
+      <x:c r="N22" s="3"/>
     </x:row>
     <x:row r="23" ht="48">
       <x:c r="A23" s="3" t="str">
@@ -14915,36 +14861,32 @@
       <x:c r="D23" s="3" t="str">
         <x:v>ARRIREAFDI</x:v>
       </x:c>
-      <x:c r="E23" s="3" t="n">
+      <x:c r="E23" s="6" t="n">
         <x:v>0.3598768533526233</x:v>
       </x:c>
-      <x:c r="F23" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G23" s="3" t="n">
+      <x:c r="F23" s="6" t="n">
         <x:v>0.3221916002899585</x:v>
       </x:c>
-      <x:c r="H23" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I23" s="3" t="n">
+      <x:c r="G23" s="6" t="n">
         <x:v>0.001053533633239567</x:v>
       </x:c>
-      <x:c r="J23" s="3" t="n">
+      <x:c r="H23" s="6" t="n">
         <x:v>0.1022641658782959</x:v>
       </x:c>
-      <x:c r="K23" s="3" t="n">
+      <x:c r="I23" s="6" t="n">
         <x:v>0.01584280468523502</x:v>
       </x:c>
-      <x:c r="L23" s="3" t="n">
+      <x:c r="J23" s="6" t="n">
         <x:v>0.01210234593600035</x:v>
       </x:c>
-      <x:c r="M23" s="3" t="n">
+      <x:c r="K23" s="6" t="n">
         <x:v>0.001633969484828413</x:v>
       </x:c>
-      <x:c r="N23" s="3" t="n">
+      <x:c r="L23" s="6" t="n">
         <x:v>0.8707876801490784</x:v>
       </x:c>
+      <x:c r="M23" s="3"/>
+      <x:c r="N23" s="3"/>
     </x:row>
     <x:row r="24" ht="48">
       <x:c r="A24" s="3" t="str">
@@ -14959,36 +14901,32 @@
       <x:c r="D24" s="3" t="str">
         <x:v>AKDRVYSLDL</x:v>
       </x:c>
-      <x:c r="E24" s="3" t="n">
+      <x:c r="E24" s="6" t="n">
         <x:v>0.3607085446908668</x:v>
       </x:c>
-      <x:c r="F24" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="3" t="n">
+      <x:c r="F24" s="6" t="n">
         <x:v>0.050398244622301</x:v>
       </x:c>
-      <x:c r="H24" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I24" s="3" t="n">
+      <x:c r="G24" s="6" t="n">
         <x:v>0.9303375482559204</x:v>
       </x:c>
-      <x:c r="J24" s="3" t="n">
+      <x:c r="H24" s="6" t="n">
         <x:v>0.9830335974693298</x:v>
       </x:c>
-      <x:c r="K24" s="3" t="n">
+      <x:c r="I24" s="6" t="n">
         <x:v>0.984717071056366</x:v>
       </x:c>
-      <x:c r="L24" s="3" t="n">
+      <x:c r="J24" s="6" t="n">
         <x:v>0.9848747849464417</x:v>
       </x:c>
-      <x:c r="M24" s="3" t="n">
+      <x:c r="K24" s="6" t="n">
         <x:v>0.9871410131454468</x:v>
       </x:c>
-      <x:c r="N24" s="3" t="n">
+      <x:c r="L24" s="6" t="n">
         <x:v>0.9897498488426208</x:v>
       </x:c>
+      <x:c r="M24" s="3"/>
+      <x:c r="N24" s="3"/>
     </x:row>
     <x:row r="25" ht="48">
       <x:c r="A25" s="3" t="str">
@@ -15003,36 +14941,32 @@
       <x:c r="D25" s="3" t="str">
         <x:v>ATLTIFHMDV</x:v>
       </x:c>
-      <x:c r="E25" s="3" t="n">
+      <x:c r="E25" s="6" t="n">
         <x:v>0.001662873645394225</x:v>
       </x:c>
-      <x:c r="F25" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G25" s="3" t="n">
+      <x:c r="F25" s="6" t="n">
         <x:v>0.001697561046006675</x:v>
       </x:c>
-      <x:c r="H25" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I25" s="3" t="n">
+      <x:c r="G25" s="6" t="n">
         <x:v>0.9806424975395203</x:v>
       </x:c>
-      <x:c r="J25" s="3" t="n">
+      <x:c r="H25" s="6" t="n">
         <x:v>0.9750483632087708</x:v>
       </x:c>
-      <x:c r="K25" s="3" t="n">
+      <x:c r="I25" s="6" t="n">
         <x:v>0.9844656586647034</x:v>
       </x:c>
-      <x:c r="L25" s="3" t="n">
+      <x:c r="J25" s="6" t="n">
         <x:v>0.972493588924408</x:v>
       </x:c>
-      <x:c r="M25" s="3" t="n">
+      <x:c r="K25" s="6" t="n">
         <x:v>0.9850349426269531</x:v>
       </x:c>
-      <x:c r="N25" s="3" t="n">
+      <x:c r="L25" s="6" t="n">
         <x:v>0.9694250822067261</x:v>
       </x:c>
+      <x:c r="M25" s="3"/>
+      <x:c r="N25" s="3"/>
     </x:row>
     <x:row r="26" ht="48">
       <x:c r="A26" s="3" t="str">
@@ -15047,36 +14981,32 @@
       <x:c r="D26" s="3" t="str">
         <x:v>ARSGVASTLDY</x:v>
       </x:c>
-      <x:c r="E26" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F26" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G26" s="3" t="n">
+      <x:c r="E26" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="6" t="n">
         <x:v>0.1013287118027675</x:v>
       </x:c>
-      <x:c r="H26" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I26" s="3" t="n">
+      <x:c r="G26" s="6" t="n">
         <x:v>0.863029956817627</x:v>
       </x:c>
-      <x:c r="J26" s="3" t="n">
+      <x:c r="H26" s="6" t="n">
         <x:v>0.9764975309371948</x:v>
       </x:c>
-      <x:c r="K26" s="3" t="n">
+      <x:c r="I26" s="6" t="n">
         <x:v>0.944616973400116</x:v>
       </x:c>
-      <x:c r="L26" s="3" t="n">
+      <x:c r="J26" s="6" t="n">
         <x:v>0.9519267678260803</x:v>
       </x:c>
-      <x:c r="M26" s="3" t="n">
+      <x:c r="K26" s="6" t="n">
         <x:v>0.8934706449508667</x:v>
       </x:c>
-      <x:c r="N26" s="3" t="n">
+      <x:c r="L26" s="6" t="n">
         <x:v>0.9817771315574646</x:v>
       </x:c>
+      <x:c r="M26" s="3"/>
+      <x:c r="N26" s="3"/>
     </x:row>
     <x:row r="27" ht="48">
       <x:c r="A27" s="3" t="str">
@@ -15091,36 +15021,32 @@
       <x:c r="D27" s="3" t="str">
         <x:v>ATDRGSLAAVD</x:v>
       </x:c>
-      <x:c r="E27" s="3" t="n">
+      <x:c r="E27" s="6" t="n">
         <x:v>0.0218483126384134</x:v>
       </x:c>
-      <x:c r="F27" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G27" s="3" t="n">
+      <x:c r="F27" s="6" t="n">
         <x:v>0.0455313190139018</x:v>
       </x:c>
-      <x:c r="H27" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I27" s="3" t="n">
+      <x:c r="G27" s="6" t="n">
         <x:v>0.05500980094075203</x:v>
       </x:c>
-      <x:c r="J27" s="3" t="n">
+      <x:c r="H27" s="6" t="n">
         <x:v>0.9342278242111206</x:v>
       </x:c>
-      <x:c r="K27" s="3" t="n">
+      <x:c r="I27" s="6" t="n">
         <x:v>0.5678543448448181</x:v>
       </x:c>
-      <x:c r="L27" s="3" t="n">
+      <x:c r="J27" s="6" t="n">
         <x:v>0.5198351740837097</x:v>
       </x:c>
-      <x:c r="M27" s="3" t="n">
+      <x:c r="K27" s="6" t="n">
         <x:v>0.7929105162620544</x:v>
       </x:c>
-      <x:c r="N27" s="3" t="n">
+      <x:c r="L27" s="6" t="n">
         <x:v>0.966439962387085</x:v>
       </x:c>
+      <x:c r="M27" s="3"/>
+      <x:c r="N27" s="3"/>
     </x:row>
     <x:row r="28" ht="48">
       <x:c r="A28" s="3" t="str">
@@ -15135,36 +15061,32 @@
       <x:c r="D28" s="3" t="str">
         <x:v>ARDVRGLPFDI</x:v>
       </x:c>
-      <x:c r="E28" s="3" t="n">
+      <x:c r="E28" s="6" t="n">
         <x:v>0.1043905054979903</x:v>
       </x:c>
-      <x:c r="F28" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G28" s="3" t="n">
+      <x:c r="F28" s="6" t="n">
         <x:v>0.1009990670862222</x:v>
       </x:c>
-      <x:c r="H28" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I28" s="3" t="n">
+      <x:c r="G28" s="6" t="n">
         <x:v>0.5650812387466431</x:v>
       </x:c>
-      <x:c r="J28" s="3" t="n">
+      <x:c r="H28" s="6" t="n">
         <x:v>0.7922407388687134</x:v>
       </x:c>
-      <x:c r="K28" s="3" t="n">
+      <x:c r="I28" s="6" t="n">
         <x:v>0.1157518550753593</x:v>
       </x:c>
-      <x:c r="L28" s="3" t="n">
+      <x:c r="J28" s="6" t="n">
         <x:v>0.952377200126648</x:v>
       </x:c>
-      <x:c r="M28" s="3" t="n">
+      <x:c r="K28" s="6" t="n">
         <x:v>0.002712443005293608</x:v>
       </x:c>
-      <x:c r="N28" s="3" t="n">
+      <x:c r="L28" s="6" t="n">
         <x:v>0.9714972972869873</x:v>
       </x:c>
+      <x:c r="M28" s="3"/>
+      <x:c r="N28" s="3"/>
     </x:row>
     <x:row r="29" ht="48">
       <x:c r="A29" s="3" t="str">
@@ -15179,36 +15101,32 @@
       <x:c r="D29" s="3" t="str">
         <x:v>ARGLVGGASDY</x:v>
       </x:c>
-      <x:c r="E29" s="3" t="n">
+      <x:c r="E29" s="6" t="n">
         <x:v>0.392898657084241</x:v>
       </x:c>
-      <x:c r="F29" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G29" s="3" t="n">
+      <x:c r="F29" s="6" t="n">
         <x:v>0.155261652635707</x:v>
       </x:c>
-      <x:c r="H29" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I29" s="3" t="n">
+      <x:c r="G29" s="6" t="n">
         <x:v>0.004438347183167934</x:v>
       </x:c>
-      <x:c r="J29" s="3" t="n">
+      <x:c r="H29" s="6" t="n">
         <x:v>0.868893563747406</x:v>
       </x:c>
-      <x:c r="K29" s="3" t="n">
+      <x:c r="I29" s="6" t="n">
         <x:v>0.7462939620018005</x:v>
       </x:c>
-      <x:c r="L29" s="3" t="n">
+      <x:c r="J29" s="6" t="n">
         <x:v>0.1530556678771973</x:v>
       </x:c>
-      <x:c r="M29" s="3" t="n">
+      <x:c r="K29" s="6" t="n">
         <x:v>0.03919404000043869</x:v>
       </x:c>
-      <x:c r="N29" s="3" t="n">
+      <x:c r="L29" s="6" t="n">
         <x:v>0.9809651970863342</x:v>
       </x:c>
+      <x:c r="M29" s="3"/>
+      <x:c r="N29" s="3"/>
     </x:row>
     <x:row r="30" ht="48">
       <x:c r="A30" s="3" t="str">
@@ -15223,36 +15141,32 @@
       <x:c r="D30" s="3" t="str">
         <x:v>ARHSQAVNAFDI</x:v>
       </x:c>
-      <x:c r="E30" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F30" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G30" s="3" t="n">
+      <x:c r="E30" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="6" t="n">
         <x:v>0.09996753264569613</x:v>
       </x:c>
-      <x:c r="H30" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I30" s="3" t="n">
+      <x:c r="G30" s="6" t="n">
         <x:v>0.3204240202903748</x:v>
       </x:c>
-      <x:c r="J30" s="3" t="n">
+      <x:c r="H30" s="6" t="n">
         <x:v>0.9834223985671997</x:v>
       </x:c>
-      <x:c r="K30" s="3" t="n">
+      <x:c r="I30" s="6" t="n">
         <x:v>0.8804805874824524</x:v>
       </x:c>
-      <x:c r="L30" s="3" t="n">
+      <x:c r="J30" s="6" t="n">
         <x:v>0.2603645026683807</x:v>
       </x:c>
-      <x:c r="M30" s="3" t="n">
+      <x:c r="K30" s="6" t="n">
         <x:v>0.09516845643520355</x:v>
       </x:c>
-      <x:c r="N30" s="3" t="n">
+      <x:c r="L30" s="6" t="n">
         <x:v>0.9969022870063782</x:v>
       </x:c>
+      <x:c r="M30" s="3"/>
+      <x:c r="N30" s="3"/>
     </x:row>
     <x:row r="31" ht="48">
       <x:c r="A31" s="3" t="str">
@@ -15267,36 +15181,32 @@
       <x:c r="D31" s="3" t="str">
         <x:v>ARGSGLAGPLDV</x:v>
       </x:c>
-      <x:c r="E31" s="3" t="n">
+      <x:c r="E31" s="6" t="n">
         <x:v>0.06197894669420327</x:v>
       </x:c>
-      <x:c r="F31" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G31" s="3" t="n">
+      <x:c r="F31" s="6" t="n">
         <x:v>0.07927494699419828</x:v>
       </x:c>
-      <x:c r="H31" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I31" s="3" t="n">
+      <x:c r="G31" s="6" t="n">
         <x:v>0.5359213948249817</x:v>
       </x:c>
-      <x:c r="J31" s="3" t="n">
+      <x:c r="H31" s="6" t="n">
         <x:v>0.7951308488845825</x:v>
       </x:c>
-      <x:c r="K31" s="3" t="n">
+      <x:c r="I31" s="6" t="n">
         <x:v>0.8337016701698303</x:v>
       </x:c>
-      <x:c r="L31" s="3" t="n">
+      <x:c r="J31" s="6" t="n">
         <x:v>0.9847656488418579</x:v>
       </x:c>
-      <x:c r="M31" s="3" t="n">
+      <x:c r="K31" s="6" t="n">
         <x:v>0.6762397885322571</x:v>
       </x:c>
-      <x:c r="N31" s="3" t="n">
+      <x:c r="L31" s="6" t="n">
         <x:v>0.9489113688468933</x:v>
       </x:c>
+      <x:c r="M31" s="3"/>
+      <x:c r="N31" s="3"/>
     </x:row>
     <x:row r="32" ht="48">
       <x:c r="A32" s="3" t="str">
@@ -15311,36 +15221,32 @@
       <x:c r="D32" s="3" t="str">
         <x:v>RLYSNYDYYFDY</x:v>
       </x:c>
-      <x:c r="E32" s="3" t="n">
+      <x:c r="E32" s="6" t="n">
         <x:v>0.004548535216796825</x:v>
       </x:c>
-      <x:c r="F32" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G32" s="3" t="n">
+      <x:c r="F32" s="6" t="n">
         <x:v>0.05512289292384143</x:v>
       </x:c>
-      <x:c r="H32" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I32" s="3" t="n">
+      <x:c r="G32" s="6" t="n">
         <x:v>0.9649269580841064</x:v>
       </x:c>
-      <x:c r="J32" s="3" t="n">
+      <x:c r="H32" s="6" t="n">
         <x:v>0.9229827523231506</x:v>
       </x:c>
-      <x:c r="K32" s="3" t="n">
+      <x:c r="I32" s="6" t="n">
         <x:v>0.9834782481193542</x:v>
       </x:c>
-      <x:c r="L32" s="3" t="n">
+      <x:c r="J32" s="6" t="n">
         <x:v>0.9875419735908508</x:v>
       </x:c>
-      <x:c r="M32" s="3" t="n">
+      <x:c r="K32" s="6" t="n">
         <x:v>0.2863708734512329</x:v>
       </x:c>
-      <x:c r="N32" s="3" t="n">
+      <x:c r="L32" s="6" t="n">
         <x:v>0.9728440046310425</x:v>
       </x:c>
+      <x:c r="M32" s="3"/>
+      <x:c r="N32" s="3"/>
     </x:row>
     <x:row r="33" ht="48">
       <x:c r="A33" s="3" t="str">
@@ -15355,36 +15261,32 @@
       <x:c r="D33" s="3" t="str">
         <x:v>ARVDILIGFTDY</x:v>
       </x:c>
-      <x:c r="E33" s="3" t="n">
+      <x:c r="E33" s="6" t="n">
         <x:v>0.01548541665657487</x:v>
       </x:c>
-      <x:c r="F33" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G33" s="3" t="n">
+      <x:c r="F33" s="6" t="n">
         <x:v>0.05128269810848035</x:v>
       </x:c>
-      <x:c r="H33" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I33" s="3" t="n">
+      <x:c r="G33" s="6" t="n">
         <x:v>0.07071401178836823</x:v>
       </x:c>
-      <x:c r="J33" s="3" t="n">
+      <x:c r="H33" s="6" t="n">
         <x:v>0.9792578816413879</x:v>
       </x:c>
-      <x:c r="K33" s="3" t="n">
+      <x:c r="I33" s="6" t="n">
         <x:v>0.001154675963334739</x:v>
       </x:c>
-      <x:c r="L33" s="3" t="n">
+      <x:c r="J33" s="6" t="n">
         <x:v>0.594519317150116</x:v>
       </x:c>
-      <x:c r="M33" s="3" t="n">
+      <x:c r="K33" s="6" t="n">
         <x:v>0.00149740744382143</x:v>
       </x:c>
-      <x:c r="N33" s="3" t="n">
+      <x:c r="L33" s="6" t="n">
         <x:v>0.9825488328933716</x:v>
       </x:c>
+      <x:c r="M33" s="3"/>
+      <x:c r="N33" s="3"/>
     </x:row>
     <x:row r="34" ht="48">
       <x:c r="A34" s="3" t="str">
@@ -15399,36 +15301,32 @@
       <x:c r="D34" s="3" t="str">
         <x:v>GRGGGVGATMVEY</x:v>
       </x:c>
-      <x:c r="E34" s="3" t="n">
+      <x:c r="E34" s="6" t="n">
         <x:v>0.02630274051575075</x:v>
       </x:c>
-      <x:c r="F34" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G34" s="3" t="n">
+      <x:c r="F34" s="6" t="n">
         <x:v>0.01040096962728193</x:v>
       </x:c>
-      <x:c r="H34" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I34" s="3" t="n">
+      <x:c r="G34" s="6" t="n">
         <x:v>0.9663528800010681</x:v>
       </x:c>
-      <x:c r="J34" s="3" t="n">
+      <x:c r="H34" s="6" t="n">
         <x:v>0.9963711500167847</x:v>
       </x:c>
-      <x:c r="K34" s="3" t="n">
+      <x:c r="I34" s="6" t="n">
         <x:v>0.9972521662712097</x:v>
       </x:c>
-      <x:c r="L34" s="3" t="n">
+      <x:c r="J34" s="6" t="n">
         <x:v>0.9969326257705688</x:v>
       </x:c>
-      <x:c r="M34" s="3" t="n">
+      <x:c r="K34" s="6" t="n">
         <x:v>0.9913837909698486</x:v>
       </x:c>
-      <x:c r="N34" s="3" t="n">
+      <x:c r="L34" s="6" t="n">
         <x:v>0.9937904477119446</x:v>
       </x:c>
+      <x:c r="M34" s="3"/>
+      <x:c r="N34" s="3"/>
     </x:row>
     <x:row r="35" ht="48">
       <x:c r="A35" s="3" t="str">
@@ -15443,36 +15341,32 @@
       <x:c r="D35" s="3" t="str">
         <x:v>ARARYGDYYYFDS</x:v>
       </x:c>
-      <x:c r="E35" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F35" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G35" s="3" t="n">
+      <x:c r="E35" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="6" t="n">
         <x:v>0.0017104521204634</x:v>
       </x:c>
-      <x:c r="H35" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I35" s="3" t="n">
+      <x:c r="G35" s="6" t="n">
         <x:v>0.004057194106280804</x:v>
       </x:c>
-      <x:c r="J35" s="3" t="n">
+      <x:c r="H35" s="6" t="n">
         <x:v>0.9047891497612</x:v>
       </x:c>
-      <x:c r="K35" s="3" t="n">
+      <x:c r="I35" s="6" t="n">
         <x:v>0.9097516536712646</x:v>
       </x:c>
-      <x:c r="L35" s="3" t="n">
+      <x:c r="J35" s="6" t="n">
         <x:v>0.8273548483848572</x:v>
       </x:c>
-      <x:c r="M35" s="3" t="n">
+      <x:c r="K35" s="6" t="n">
         <x:v>0.3801979124546051</x:v>
       </x:c>
-      <x:c r="N35" s="3" t="n">
+      <x:c r="L35" s="6" t="n">
         <x:v>0.7415006160736084</x:v>
       </x:c>
+      <x:c r="M35" s="3"/>
+      <x:c r="N35" s="3"/>
     </x:row>
     <x:row r="36" ht="48">
       <x:c r="A36" s="3" t="str">
@@ -15487,36 +15381,32 @@
       <x:c r="D36" s="3" t="str">
         <x:v>TRDRSEYSSPSLY</x:v>
       </x:c>
-      <x:c r="E36" s="3" t="n">
+      <x:c r="E36" s="6" t="n">
         <x:v>0.02069667989078888</x:v>
       </x:c>
-      <x:c r="F36" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G36" s="3" t="n">
+      <x:c r="F36" s="6" t="n">
         <x:v>0.09986307476550832</x:v>
       </x:c>
-      <x:c r="H36" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I36" s="3" t="n">
+      <x:c r="G36" s="6" t="n">
         <x:v>0.02545022033154964</x:v>
       </x:c>
-      <x:c r="J36" s="3" t="n">
+      <x:c r="H36" s="6" t="n">
         <x:v>0.6770957112312317</x:v>
       </x:c>
-      <x:c r="K36" s="3" t="n">
+      <x:c r="I36" s="6" t="n">
         <x:v>0.8805353045463562</x:v>
       </x:c>
-      <x:c r="L36" s="3" t="n">
+      <x:c r="J36" s="6" t="n">
         <x:v>0.8108598589897156</x:v>
       </x:c>
-      <x:c r="M36" s="3" t="n">
+      <x:c r="K36" s="6" t="n">
         <x:v>0.007658916991204023</x:v>
       </x:c>
-      <x:c r="N36" s="3" t="n">
+      <x:c r="L36" s="6" t="n">
         <x:v>0.9880444407463074</x:v>
       </x:c>
+      <x:c r="M36" s="3"/>
+      <x:c r="N36" s="3"/>
     </x:row>
     <x:row r="37" ht="48">
       <x:c r="A37" s="3" t="str">
@@ -15531,36 +15421,32 @@
       <x:c r="D37" s="3" t="str">
         <x:v>AVGFNFHYYYMDV</x:v>
       </x:c>
-      <x:c r="E37" s="3" t="n">
+      <x:c r="E37" s="6" t="n">
         <x:v>0.02597193469826303</x:v>
       </x:c>
-      <x:c r="F37" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G37" s="3" t="n">
+      <x:c r="F37" s="6" t="n">
         <x:v>0.0828922951743861</x:v>
       </x:c>
-      <x:c r="H37" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I37" s="3" t="n">
+      <x:c r="G37" s="6" t="n">
         <x:v>0.4562017023563385</x:v>
       </x:c>
-      <x:c r="J37" s="3" t="n">
+      <x:c r="H37" s="6" t="n">
         <x:v>0.5680927634239197</x:v>
       </x:c>
-      <x:c r="K37" s="3" t="n">
+      <x:c r="I37" s="6" t="n">
         <x:v>0.9489765167236328</x:v>
       </x:c>
-      <x:c r="L37" s="3" t="n">
+      <x:c r="J37" s="6" t="n">
         <x:v>0.9945995807647705</x:v>
       </x:c>
-      <x:c r="M37" s="3" t="n">
+      <x:c r="K37" s="6" t="n">
         <x:v>0.9879797697067261</x:v>
       </x:c>
-      <x:c r="N37" s="3" t="n">
+      <x:c r="L37" s="6" t="n">
         <x:v>0.9929074048995972</x:v>
       </x:c>
+      <x:c r="M37" s="3"/>
+      <x:c r="N37" s="3"/>
     </x:row>
     <x:row r="38" ht="48">
       <x:c r="A38" s="3" t="str">
@@ -15575,36 +15461,32 @@
       <x:c r="D38" s="3" t="str">
         <x:v>AGHSRVYGSPAFDF</x:v>
       </x:c>
-      <x:c r="E38" s="3" t="n">
+      <x:c r="E38" s="6" t="n">
         <x:v>0.0104231533742725</x:v>
       </x:c>
-      <x:c r="F38" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G38" s="3" t="n">
+      <x:c r="F38" s="6" t="n">
         <x:v>0.1002396255633695</x:v>
       </x:c>
-      <x:c r="H38" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I38" s="3" t="n">
+      <x:c r="G38" s="6" t="n">
         <x:v>0.004038793500512838</x:v>
       </x:c>
-      <x:c r="J38" s="3" t="n">
+      <x:c r="H38" s="6" t="n">
         <x:v>0.1940126866102219</x:v>
       </x:c>
-      <x:c r="K38" s="3" t="n">
+      <x:c r="I38" s="6" t="n">
         <x:v>0.01995637081563473</x:v>
       </x:c>
-      <x:c r="L38" s="3" t="n">
+      <x:c r="J38" s="6" t="n">
         <x:v>0.8666971325874329</x:v>
       </x:c>
-      <x:c r="M38" s="3" t="n">
+      <x:c r="K38" s="6" t="n">
         <x:v>0.00165255053434521</x:v>
       </x:c>
-      <x:c r="N38" s="3" t="n">
+      <x:c r="L38" s="6" t="n">
         <x:v>0.8834707736968994</x:v>
       </x:c>
+      <x:c r="M38" s="3"/>
+      <x:c r="N38" s="3"/>
     </x:row>
     <x:row r="39" ht="48">
       <x:c r="A39" s="3" t="str">
@@ -15619,36 +15501,32 @@
       <x:c r="D39" s="3" t="str">
         <x:v>ARNIVPARSKWFDP</x:v>
       </x:c>
-      <x:c r="E39" s="3" t="n">
+      <x:c r="E39" s="6" t="n">
         <x:v>0.1007851472246015</x:v>
       </x:c>
-      <x:c r="F39" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G39" s="3" t="n">
+      <x:c r="F39" s="6" t="n">
         <x:v>0.09994214595420703</x:v>
       </x:c>
-      <x:c r="H39" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I39" s="3" t="n">
+      <x:c r="G39" s="6" t="n">
         <x:v>0.003808613168075681</x:v>
       </x:c>
-      <x:c r="J39" s="3" t="n">
+      <x:c r="H39" s="6" t="n">
         <x:v>0.9843921661376953</x:v>
       </x:c>
-      <x:c r="K39" s="3" t="n">
+      <x:c r="I39" s="6" t="n">
         <x:v>0.8751562237739563</x:v>
       </x:c>
-      <x:c r="L39" s="3" t="n">
+      <x:c r="J39" s="6" t="n">
         <x:v>0.9960846900939941</x:v>
       </x:c>
-      <x:c r="M39" s="3" t="n">
+      <x:c r="K39" s="6" t="n">
         <x:v>0.00959615595638752</x:v>
       </x:c>
-      <x:c r="N39" s="3" t="n">
+      <x:c r="L39" s="6" t="n">
         <x:v>0.9492496252059937</x:v>
       </x:c>
+      <x:c r="M39" s="3"/>
+      <x:c r="N39" s="3"/>
     </x:row>
     <x:row r="40" ht="48">
       <x:c r="A40" s="3" t="str">
@@ -15663,36 +15541,32 @@
       <x:c r="D40" s="3" t="str">
         <x:v>ARLKSRSSWAAFDI</x:v>
       </x:c>
-      <x:c r="E40" s="3" t="n">
+      <x:c r="E40" s="6" t="n">
         <x:v>0.4272962431747538</x:v>
       </x:c>
-      <x:c r="F40" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G40" s="3" t="n">
+      <x:c r="F40" s="6" t="n">
         <x:v>0.1235305134865315</x:v>
       </x:c>
-      <x:c r="H40" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I40" s="3" t="n">
+      <x:c r="G40" s="6" t="n">
         <x:v>0.001493459334596992</x:v>
       </x:c>
-      <x:c r="J40" s="3" t="n">
+      <x:c r="H40" s="6" t="n">
         <x:v>0.3687694668769836</x:v>
       </x:c>
-      <x:c r="K40" s="3" t="n">
+      <x:c r="I40" s="6" t="n">
         <x:v>0.6843324303627014</x:v>
       </x:c>
-      <x:c r="L40" s="3" t="n">
+      <x:c r="J40" s="6" t="n">
         <x:v>0.00453411228954792</x:v>
       </x:c>
-      <x:c r="M40" s="3" t="n">
+      <x:c r="K40" s="6" t="n">
         <x:v>0.05648667737841606</x:v>
       </x:c>
-      <x:c r="N40" s="3" t="n">
+      <x:c r="L40" s="6" t="n">
         <x:v>0.9567399621009827</x:v>
       </x:c>
+      <x:c r="M40" s="3"/>
+      <x:c r="N40" s="3"/>
     </x:row>
     <x:row r="41" ht="48">
       <x:c r="A41" s="3" t="str">
@@ -15707,36 +15581,32 @@
       <x:c r="D41" s="3" t="str">
         <x:v>ARHSRGGSSYWFDP</x:v>
       </x:c>
-      <x:c r="E41" s="3" t="n">
+      <x:c r="E41" s="6" t="n">
         <x:v>0.1030021570626465</x:v>
       </x:c>
-      <x:c r="F41" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G41" s="3" t="n">
+      <x:c r="F41" s="6" t="n">
         <x:v>0.1033337941339385</x:v>
       </x:c>
-      <x:c r="H41" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I41" s="3" t="n">
+      <x:c r="G41" s="6" t="n">
         <x:v>0.9261426329612732</x:v>
       </x:c>
-      <x:c r="J41" s="3" t="n">
+      <x:c r="H41" s="6" t="n">
         <x:v>0.9872450232505798</x:v>
       </x:c>
-      <x:c r="K41" s="3" t="n">
+      <x:c r="I41" s="6" t="n">
         <x:v>0.9776304364204407</x:v>
       </x:c>
-      <x:c r="L41" s="3" t="n">
+      <x:c r="J41" s="6" t="n">
         <x:v>0.8501009941101074</x:v>
       </x:c>
-      <x:c r="M41" s="3" t="n">
+      <x:c r="K41" s="6" t="n">
         <x:v>0.8910120725631714</x:v>
       </x:c>
-      <x:c r="N41" s="3" t="n">
+      <x:c r="L41" s="6" t="n">
         <x:v>0.9761358499526978</x:v>
       </x:c>
+      <x:c r="M41" s="3"/>
+      <x:c r="N41" s="3"/>
     </x:row>
     <x:row r="42" ht="48">
       <x:c r="A42" s="3" t="str">
@@ -15751,36 +15621,32 @@
       <x:c r="D42" s="3" t="str">
         <x:v>AKPRGENIGRLGVDY</x:v>
       </x:c>
-      <x:c r="E42" s="3" t="n">
+      <x:c r="E42" s="6" t="n">
         <x:v>0.000958933099813275</x:v>
       </x:c>
-      <x:c r="F42" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G42" s="3" t="n">
+      <x:c r="F42" s="6" t="n">
         <x:v>0.0896067227505862</x:v>
       </x:c>
-      <x:c r="H42" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I42" s="3" t="n">
+      <x:c r="G42" s="6" t="n">
         <x:v>0.9084597229957581</x:v>
       </x:c>
-      <x:c r="J42" s="3" t="n">
+      <x:c r="H42" s="6" t="n">
         <x:v>0.9878331422805786</x:v>
       </x:c>
-      <x:c r="K42" s="3" t="n">
+      <x:c r="I42" s="6" t="n">
         <x:v>0.6161493062973022</x:v>
       </x:c>
-      <x:c r="L42" s="3" t="n">
+      <x:c r="J42" s="6" t="n">
         <x:v>0.9463859796524048</x:v>
       </x:c>
-      <x:c r="M42" s="3" t="n">
+      <x:c r="K42" s="6" t="n">
         <x:v>0.008890099823474884</x:v>
       </x:c>
-      <x:c r="N42" s="3" t="n">
+      <x:c r="L42" s="6" t="n">
         <x:v>0.9566783308982849</x:v>
       </x:c>
+      <x:c r="M42" s="3"/>
+      <x:c r="N42" s="3"/>
     </x:row>
     <x:row r="43" ht="48">
       <x:c r="A43" s="3" t="str">
@@ -15795,36 +15661,32 @@
       <x:c r="D43" s="3" t="str">
         <x:v>ARYDYIGRLKASFGL</x:v>
       </x:c>
-      <x:c r="E43" s="3" t="n">
+      <x:c r="E43" s="6" t="n">
         <x:v>0.0088968631310454</x:v>
       </x:c>
-      <x:c r="F43" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G43" s="3" t="n">
+      <x:c r="F43" s="6" t="n">
         <x:v>0.05690899447272203</x:v>
       </x:c>
-      <x:c r="H43" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I43" s="3" t="n">
+      <x:c r="G43" s="6" t="n">
         <x:v>0.78902268409729</x:v>
       </x:c>
-      <x:c r="J43" s="3" t="n">
+      <x:c r="H43" s="6" t="n">
         <x:v>0.7103015184402466</x:v>
       </x:c>
-      <x:c r="K43" s="3" t="n">
+      <x:c r="I43" s="6" t="n">
         <x:v>0.9888594150543213</x:v>
       </x:c>
-      <x:c r="L43" s="3" t="n">
+      <x:c r="J43" s="6" t="n">
         <x:v>0.995048463344574</x:v>
       </x:c>
-      <x:c r="M43" s="3" t="n">
+      <x:c r="K43" s="6" t="n">
         <x:v>0.3339917361736298</x:v>
       </x:c>
-      <x:c r="N43" s="3" t="n">
+      <x:c r="L43" s="6" t="n">
         <x:v>0.993130624294281</x:v>
       </x:c>
+      <x:c r="M43" s="3"/>
+      <x:c r="N43" s="3"/>
     </x:row>
     <x:row r="44" ht="48">
       <x:c r="A44" s="3" t="str">
@@ -15839,36 +15701,32 @@
       <x:c r="D44" s="3" t="str">
         <x:v>AKDTDFSGYYYYMDV</x:v>
       </x:c>
-      <x:c r="E44" s="3" t="n">
+      <x:c r="E44" s="6" t="n">
         <x:v>0.005883210322091725</x:v>
       </x:c>
-      <x:c r="F44" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G44" s="3" t="n">
+      <x:c r="F44" s="6" t="n">
         <x:v>0.04020656781642423</x:v>
       </x:c>
-      <x:c r="H44" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I44" s="3" t="n">
+      <x:c r="G44" s="6" t="n">
         <x:v>0.9772573709487915</x:v>
       </x:c>
-      <x:c r="J44" s="3" t="n">
+      <x:c r="H44" s="6" t="n">
         <x:v>0.9948511719703674</x:v>
       </x:c>
-      <x:c r="K44" s="3" t="n">
+      <x:c r="I44" s="6" t="n">
         <x:v>0.9873936176300049</x:v>
       </x:c>
-      <x:c r="L44" s="3" t="n">
+      <x:c r="J44" s="6" t="n">
         <x:v>0.9979404807090759</x:v>
       </x:c>
-      <x:c r="M44" s="3" t="n">
+      <x:c r="K44" s="6" t="n">
         <x:v>0.9957102537155151</x:v>
       </x:c>
-      <x:c r="N44" s="3" t="n">
+      <x:c r="L44" s="6" t="n">
         <x:v>0.9936119914054871</x:v>
       </x:c>
+      <x:c r="M44" s="3"/>
+      <x:c r="N44" s="3"/>
     </x:row>
     <x:row r="45" ht="48">
       <x:c r="A45" s="3" t="str">
@@ -15883,36 +15741,32 @@
       <x:c r="D45" s="3" t="str">
         <x:v>AIASMIADWYYGMDV</x:v>
       </x:c>
-      <x:c r="E45" s="3" t="n">
+      <x:c r="E45" s="6" t="n">
         <x:v>0.01082678117690505</x:v>
       </x:c>
-      <x:c r="F45" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G45" s="3" t="n">
+      <x:c r="F45" s="6" t="n">
         <x:v>0.0561732329103278</x:v>
       </x:c>
-      <x:c r="H45" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I45" s="3" t="n">
+      <x:c r="G45" s="6" t="n">
         <x:v>0.9288750290870667</x:v>
       </x:c>
-      <x:c r="J45" s="3" t="n">
+      <x:c r="H45" s="6" t="n">
         <x:v>0.9355222582817078</x:v>
       </x:c>
-      <x:c r="K45" s="3" t="n">
+      <x:c r="I45" s="6" t="n">
         <x:v>0.9513806700706482</x:v>
       </x:c>
-      <x:c r="L45" s="3" t="n">
+      <x:c r="J45" s="6" t="n">
         <x:v>0.9715391397476196</x:v>
       </x:c>
-      <x:c r="M45" s="3" t="n">
+      <x:c r="K45" s="6" t="n">
         <x:v>0.8854801654815674</x:v>
       </x:c>
-      <x:c r="N45" s="3" t="n">
+      <x:c r="L45" s="6" t="n">
         <x:v>0.9454650282859802</x:v>
       </x:c>
+      <x:c r="M45" s="3"/>
+      <x:c r="N45" s="3"/>
     </x:row>
     <x:row r="46" ht="48">
       <x:c r="A46" s="3" t="str">
@@ -15927,36 +15781,32 @@
       <x:c r="D46" s="3" t="str">
         <x:v>ARAQWDIVSPGNAFDI</x:v>
       </x:c>
-      <x:c r="E46" s="3" t="n">
+      <x:c r="E46" s="6" t="n">
         <x:v>0.1706331548413487</x:v>
       </x:c>
-      <x:c r="F46" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G46" s="3" t="n">
+      <x:c r="F46" s="6" t="n">
         <x:v>0.09436008080370027</x:v>
       </x:c>
-      <x:c r="H46" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I46" s="3" t="n">
+      <x:c r="G46" s="6" t="n">
         <x:v>0.3868951201438904</x:v>
       </x:c>
-      <x:c r="J46" s="3" t="n">
+      <x:c r="H46" s="6" t="n">
         <x:v>0.9397905468940735</x:v>
       </x:c>
-      <x:c r="K46" s="3" t="n">
+      <x:c r="I46" s="6" t="n">
         <x:v>0.958013117313385</x:v>
       </x:c>
-      <x:c r="L46" s="3" t="n">
+      <x:c r="J46" s="6" t="n">
         <x:v>0.9807475209236145</x:v>
       </x:c>
-      <x:c r="M46" s="3" t="n">
+      <x:c r="K46" s="6" t="n">
         <x:v>0.9640437960624695</x:v>
       </x:c>
-      <x:c r="N46" s="3" t="n">
+      <x:c r="L46" s="6" t="n">
         <x:v>0.9731386303901672</x:v>
       </x:c>
+      <x:c r="M46" s="3"/>
+      <x:c r="N46" s="3"/>
     </x:row>
     <x:row r="47" ht="48">
       <x:c r="A47" s="3" t="str">
@@ -15971,36 +15821,32 @@
       <x:c r="D47" s="3" t="str">
         <x:v>ARTLRATFVTGGQVHV</x:v>
       </x:c>
-      <x:c r="E47" s="3" t="n">
+      <x:c r="E47" s="6" t="n">
         <x:v>0.05828516528812075</x:v>
       </x:c>
-      <x:c r="F47" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G47" s="3" t="n">
+      <x:c r="F47" s="6" t="n">
         <x:v>0.067591563066923</x:v>
       </x:c>
-      <x:c r="H47" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I47" s="3" t="n">
+      <x:c r="G47" s="6" t="n">
         <x:v>0.8945560455322266</x:v>
       </x:c>
-      <x:c r="J47" s="3" t="n">
+      <x:c r="H47" s="6" t="n">
         <x:v>0.655323326587677</x:v>
       </x:c>
-      <x:c r="K47" s="3" t="n">
+      <x:c r="I47" s="6" t="n">
         <x:v>0.804268479347229</x:v>
       </x:c>
-      <x:c r="L47" s="3" t="n">
+      <x:c r="J47" s="6" t="n">
         <x:v>0.4923603236675262</x:v>
       </x:c>
-      <x:c r="M47" s="3" t="n">
+      <x:c r="K47" s="6" t="n">
         <x:v>0.9745518565177917</x:v>
       </x:c>
-      <x:c r="N47" s="3" t="n">
+      <x:c r="L47" s="6" t="n">
         <x:v>0.4236648678779602</x:v>
       </x:c>
+      <x:c r="M47" s="3"/>
+      <x:c r="N47" s="3"/>
     </x:row>
     <x:row r="48" ht="48">
       <x:c r="A48" s="3" t="str">
@@ -16015,36 +15861,32 @@
       <x:c r="D48" s="3" t="str">
         <x:v>AKEFGGAISGKDAFDA</x:v>
       </x:c>
-      <x:c r="E48" s="3" t="n">
+      <x:c r="E48" s="6" t="n">
         <x:v>0.135282834725081</x:v>
       </x:c>
-      <x:c r="F48" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G48" s="3" t="n">
+      <x:c r="F48" s="6" t="n">
         <x:v>0.1207493422352657</x:v>
       </x:c>
-      <x:c r="H48" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I48" s="3" t="n">
+      <x:c r="G48" s="6" t="n">
         <x:v>0.03443407639861107</x:v>
       </x:c>
-      <x:c r="J48" s="3" t="n">
+      <x:c r="H48" s="6" t="n">
         <x:v>0.005220284219831228</x:v>
       </x:c>
-      <x:c r="K48" s="3" t="n">
+      <x:c r="I48" s="6" t="n">
         <x:v>0.00867093913257122</x:v>
       </x:c>
-      <x:c r="L48" s="3" t="n">
+      <x:c r="J48" s="6" t="n">
         <x:v>0.9644649028778076</x:v>
       </x:c>
-      <x:c r="M48" s="3" t="n">
+      <x:c r="K48" s="6" t="n">
         <x:v>0.001469284063205123</x:v>
       </x:c>
-      <x:c r="N48" s="3" t="n">
+      <x:c r="L48" s="6" t="n">
         <x:v>0.9938517808914185</x:v>
       </x:c>
+      <x:c r="M48" s="3"/>
+      <x:c r="N48" s="3"/>
     </x:row>
     <x:row r="49" ht="48">
       <x:c r="A49" s="3" t="str">
@@ -16059,36 +15901,32 @@
       <x:c r="D49" s="3" t="str">
         <x:v>ARGGWDYEDYVPNLDY</x:v>
       </x:c>
-      <x:c r="E49" s="3" t="n">
+      <x:c r="E49" s="6" t="n">
         <x:v>0.01102874047703582</x:v>
       </x:c>
-      <x:c r="F49" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G49" s="3" t="n">
+      <x:c r="F49" s="6" t="n">
         <x:v>0.05443771625274388</x:v>
       </x:c>
-      <x:c r="H49" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I49" s="3" t="n">
+      <x:c r="G49" s="6" t="n">
         <x:v>0.9753789305686951</x:v>
       </x:c>
-      <x:c r="J49" s="3" t="n">
+      <x:c r="H49" s="6" t="n">
         <x:v>0.9284682869911194</x:v>
       </x:c>
-      <x:c r="K49" s="3" t="n">
+      <x:c r="I49" s="6" t="n">
         <x:v>0.8008458018302917</x:v>
       </x:c>
-      <x:c r="L49" s="3" t="n">
+      <x:c r="J49" s="6" t="n">
         <x:v>0.8961930274963379</x:v>
       </x:c>
-      <x:c r="M49" s="3" t="n">
+      <x:c r="K49" s="6" t="n">
         <x:v>0.6090403199195862</x:v>
       </x:c>
-      <x:c r="N49" s="3" t="n">
+      <x:c r="L49" s="6" t="n">
         <x:v>0.9968966245651245</x:v>
       </x:c>
+      <x:c r="M49" s="3"/>
+      <x:c r="N49" s="3"/>
     </x:row>
     <x:row r="50" ht="48">
       <x:c r="A50" s="3" t="str">
@@ -16103,36 +15941,32 @@
       <x:c r="D50" s="3" t="str">
         <x:v>ARRLTLVAHSFHNYMDV</x:v>
       </x:c>
-      <x:c r="E50" s="3" t="n">
+      <x:c r="E50" s="6" t="n">
         <x:v>0.001221463668591275</x:v>
       </x:c>
-      <x:c r="F50" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G50" s="3" t="n">
+      <x:c r="F50" s="6" t="n">
         <x:v>0.058997481079426</x:v>
       </x:c>
-      <x:c r="H50" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I50" s="3" t="n">
+      <x:c r="G50" s="6" t="n">
         <x:v>0.0518692210316658</x:v>
       </x:c>
-      <x:c r="J50" s="3" t="n">
+      <x:c r="H50" s="6" t="n">
         <x:v>0.9429615139961243</x:v>
       </x:c>
-      <x:c r="K50" s="3" t="n">
+      <x:c r="I50" s="6" t="n">
         <x:v>0.6593679189682007</x:v>
       </x:c>
-      <x:c r="L50" s="3" t="n">
+      <x:c r="J50" s="6" t="n">
         <x:v>0.9739511609077454</x:v>
       </x:c>
-      <x:c r="M50" s="3" t="n">
+      <x:c r="K50" s="6" t="n">
         <x:v>0.9737512469291687</x:v>
       </x:c>
-      <x:c r="N50" s="3" t="n">
+      <x:c r="L50" s="6" t="n">
         <x:v>0.9581888318061829</x:v>
       </x:c>
+      <x:c r="M50" s="3"/>
+      <x:c r="N50" s="3"/>
     </x:row>
     <x:row r="51" ht="48">
       <x:c r="A51" s="3" t="str">
@@ -16147,36 +15981,32 @@
       <x:c r="D51" s="3" t="str">
         <x:v>ARVKEQWLSRGGNSFDL</x:v>
       </x:c>
-      <x:c r="E51" s="3" t="n">
+      <x:c r="E51" s="6" t="n">
         <x:v>0.1160323821956157</x:v>
       </x:c>
-      <x:c r="F51" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G51" s="3" t="n">
+      <x:c r="F51" s="6" t="n">
         <x:v>0.1423002741124258</x:v>
       </x:c>
-      <x:c r="H51" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I51" s="3" t="n">
+      <x:c r="G51" s="6" t="n">
         <x:v>0.001765485503710806</x:v>
       </x:c>
-      <x:c r="J51" s="3" t="n">
+      <x:c r="H51" s="6" t="n">
         <x:v>0.7279897332191467</x:v>
       </x:c>
-      <x:c r="K51" s="3" t="n">
+      <x:c r="I51" s="6" t="n">
         <x:v>0.001967130461707711</x:v>
       </x:c>
-      <x:c r="L51" s="3" t="n">
+      <x:c r="J51" s="6" t="n">
         <x:v>0.004497026093304157</x:v>
       </x:c>
-      <x:c r="M51" s="3" t="n">
+      <x:c r="K51" s="6" t="n">
         <x:v>0.001827026251703501</x:v>
       </x:c>
-      <x:c r="N51" s="3" t="n">
+      <x:c r="L51" s="6" t="n">
         <x:v>0.9776911735534668</x:v>
       </x:c>
+      <x:c r="M51" s="3"/>
+      <x:c r="N51" s="3"/>
     </x:row>
     <x:row r="52" ht="48">
       <x:c r="A52" s="3" t="str">
@@ -16191,36 +16021,32 @@
       <x:c r="D52" s="3" t="str">
         <x:v>ARRSDDYGDYYGRYFDY</x:v>
       </x:c>
-      <x:c r="E52" s="3" t="n">
+      <x:c r="E52" s="6" t="n">
         <x:v>0.0226941182746505</x:v>
       </x:c>
-      <x:c r="F52" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G52" s="3" t="n">
+      <x:c r="F52" s="6" t="n">
         <x:v>0.0399883868839978</x:v>
       </x:c>
-      <x:c r="H52" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I52" s="3" t="n">
+      <x:c r="G52" s="6" t="n">
         <x:v>0.8829199075698853</x:v>
       </x:c>
-      <x:c r="J52" s="3" t="n">
+      <x:c r="H52" s="6" t="n">
         <x:v>0.983187735080719</x:v>
       </x:c>
-      <x:c r="K52" s="3" t="n">
+      <x:c r="I52" s="6" t="n">
         <x:v>0.9793638586997986</x:v>
       </x:c>
-      <x:c r="L52" s="3" t="n">
+      <x:c r="J52" s="6" t="n">
         <x:v>0.9931910634040833</x:v>
       </x:c>
-      <x:c r="M52" s="3" t="n">
+      <x:c r="K52" s="6" t="n">
         <x:v>0.8554579019546509</x:v>
       </x:c>
-      <x:c r="N52" s="3" t="n">
+      <x:c r="L52" s="6" t="n">
         <x:v>0.9952768087387085</x:v>
       </x:c>
+      <x:c r="M52" s="3"/>
+      <x:c r="N52" s="3"/>
     </x:row>
     <x:row r="53" ht="48">
       <x:c r="A53" s="3" t="str">
@@ -16235,36 +16061,32 @@
       <x:c r="D53" s="3" t="str">
         <x:v>ARVESVVVPIAGNWFDS</x:v>
       </x:c>
-      <x:c r="E53" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F53" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G53" s="3" t="n">
+      <x:c r="E53" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F53" s="6" t="n">
         <x:v>0.05283114295137907</x:v>
       </x:c>
-      <x:c r="H53" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I53" s="3" t="n">
+      <x:c r="G53" s="6" t="n">
         <x:v>0.963359534740448</x:v>
       </x:c>
-      <x:c r="J53" s="3" t="n">
+      <x:c r="H53" s="6" t="n">
         <x:v>0.9955711960792542</x:v>
       </x:c>
-      <x:c r="K53" s="3" t="n">
+      <x:c r="I53" s="6" t="n">
         <x:v>0.9959781169891357</x:v>
       </x:c>
-      <x:c r="L53" s="3" t="n">
+      <x:c r="J53" s="6" t="n">
         <x:v>0.9976599216461182</x:v>
       </x:c>
-      <x:c r="M53" s="3" t="n">
+      <x:c r="K53" s="6" t="n">
         <x:v>0.9090989828109741</x:v>
       </x:c>
-      <x:c r="N53" s="3" t="n">
+      <x:c r="L53" s="6" t="n">
         <x:v>0.9882133603096008</x:v>
       </x:c>
+      <x:c r="M53" s="3"/>
+      <x:c r="N53" s="3"/>
     </x:row>
     <x:row r="54" ht="48">
       <x:c r="A54" s="3" t="str">
@@ -16279,36 +16101,32 @@
       <x:c r="D54" s="3" t="str">
         <x:v>AKFAPFWTTTDYDYYMDV</x:v>
       </x:c>
-      <x:c r="E54" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F54" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G54" s="3" t="n">
+      <x:c r="E54" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F54" s="6" t="n">
         <x:v>0.04126606859305582</x:v>
       </x:c>
-      <x:c r="H54" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I54" s="3" t="n">
+      <x:c r="G54" s="6" t="n">
         <x:v>0.9847062230110168</x:v>
       </x:c>
-      <x:c r="J54" s="3" t="n">
+      <x:c r="H54" s="6" t="n">
         <x:v>0.9933638572692871</x:v>
       </x:c>
-      <x:c r="K54" s="3" t="n">
+      <x:c r="I54" s="6" t="n">
         <x:v>0.5727962255477905</x:v>
       </x:c>
-      <x:c r="L54" s="3" t="n">
+      <x:c r="J54" s="6" t="n">
         <x:v>0.9822306036949158</x:v>
       </x:c>
-      <x:c r="M54" s="3" t="n">
+      <x:c r="K54" s="6" t="n">
         <x:v>0.01317047514021397</x:v>
       </x:c>
-      <x:c r="N54" s="3" t="n">
+      <x:c r="L54" s="6" t="n">
         <x:v>0.9930960536003113</x:v>
       </x:c>
+      <x:c r="M54" s="3"/>
+      <x:c r="N54" s="3"/>
     </x:row>
     <x:row r="55" ht="48">
       <x:c r="A55" s="3" t="str">
@@ -16323,36 +16141,32 @@
       <x:c r="D55" s="3" t="str">
         <x:v>ARDNLQMGILTAIGVVDH</x:v>
       </x:c>
-      <x:c r="E55" s="3" t="n">
+      <x:c r="E55" s="6" t="n">
         <x:v>0.04709365191547785</x:v>
       </x:c>
-      <x:c r="F55" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G55" s="3" t="n">
+      <x:c r="F55" s="6" t="n">
         <x:v>0.0998675922792831</x:v>
       </x:c>
-      <x:c r="H55" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I55" s="3" t="n">
+      <x:c r="G55" s="6" t="n">
         <x:v>0.9671851992607117</x:v>
       </x:c>
-      <x:c r="J55" s="3" t="n">
+      <x:c r="H55" s="6" t="n">
         <x:v>0.994243323802948</x:v>
       </x:c>
-      <x:c r="K55" s="3" t="n">
+      <x:c r="I55" s="6" t="n">
         <x:v>0.8232651948928833</x:v>
       </x:c>
-      <x:c r="L55" s="3" t="n">
+      <x:c r="J55" s="6" t="n">
         <x:v>0.9973770380020142</x:v>
       </x:c>
-      <x:c r="M55" s="3" t="n">
+      <x:c r="K55" s="6" t="n">
         <x:v>0.8630475401878357</x:v>
       </x:c>
-      <x:c r="N55" s="3" t="n">
+      <x:c r="L55" s="6" t="n">
         <x:v>0.9945514798164368</x:v>
       </x:c>
+      <x:c r="M55" s="3"/>
+      <x:c r="N55" s="3"/>
     </x:row>
     <x:row r="56" ht="48">
       <x:c r="A56" s="3" t="str">
@@ -16367,36 +16181,32 @@
       <x:c r="D56" s="3" t="str">
         <x:v>VRDRNYHDRRTYYDVLDV</x:v>
       </x:c>
-      <x:c r="E56" s="3" t="n">
+      <x:c r="E56" s="6" t="n">
         <x:v>0.09126931301810755</x:v>
       </x:c>
-      <x:c r="F56" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G56" s="3" t="n">
+      <x:c r="F56" s="6" t="n">
         <x:v>0.09976554285527292</x:v>
       </x:c>
-      <x:c r="H56" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I56" s="3" t="n">
+      <x:c r="G56" s="6" t="n">
         <x:v>0.04042317345738411</x:v>
       </x:c>
-      <x:c r="J56" s="3" t="n">
+      <x:c r="H56" s="6" t="n">
         <x:v>0.9400094747543335</x:v>
       </x:c>
-      <x:c r="K56" s="3" t="n">
+      <x:c r="I56" s="6" t="n">
         <x:v>0.9851778149604797</x:v>
       </x:c>
-      <x:c r="L56" s="3" t="n">
+      <x:c r="J56" s="6" t="n">
         <x:v>0.9882402420043945</x:v>
       </x:c>
-      <x:c r="M56" s="3" t="n">
+      <x:c r="K56" s="6" t="n">
         <x:v>0.002808023942634463</x:v>
       </x:c>
-      <x:c r="N56" s="3" t="n">
+      <x:c r="L56" s="6" t="n">
         <x:v>0.8598389029502869</x:v>
       </x:c>
+      <x:c r="M56" s="3"/>
+      <x:c r="N56" s="3"/>
     </x:row>
     <x:row r="57" ht="48">
       <x:c r="A57" s="3" t="str">
@@ -16411,36 +16221,32 @@
       <x:c r="D57" s="3" t="str">
         <x:v>ARDWGGYSHFAYYSYMDV</x:v>
       </x:c>
-      <x:c r="E57" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F57" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G57" s="3" t="n">
+      <x:c r="E57" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F57" s="6" t="n">
         <x:v>0.05911826661421965</x:v>
       </x:c>
-      <x:c r="H57" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I57" s="3" t="n">
+      <x:c r="G57" s="6" t="n">
         <x:v>0.9195085167884827</x:v>
       </x:c>
-      <x:c r="J57" s="3" t="n">
+      <x:c r="H57" s="6" t="n">
         <x:v>0.9717584848403931</x:v>
       </x:c>
-      <x:c r="K57" s="3" t="n">
+      <x:c r="I57" s="6" t="n">
         <x:v>0.975941002368927</x:v>
       </x:c>
-      <x:c r="L57" s="3" t="n">
+      <x:c r="J57" s="6" t="n">
         <x:v>0.9873493313789368</x:v>
       </x:c>
-      <x:c r="M57" s="3" t="n">
+      <x:c r="K57" s="6" t="n">
         <x:v>0.9891462326049805</x:v>
       </x:c>
-      <x:c r="N57" s="3" t="n">
+      <x:c r="L57" s="6" t="n">
         <x:v>0.9941185712814331</x:v>
       </x:c>
+      <x:c r="M57" s="3"/>
+      <x:c r="N57" s="3"/>
     </x:row>
     <x:row r="58" ht="48">
       <x:c r="A58" s="3" t="str">
@@ -16455,36 +16261,32 @@
       <x:c r="D58" s="3" t="str">
         <x:v>ARRADYYDSSGDYLDAFDI</x:v>
       </x:c>
-      <x:c r="E58" s="3" t="n">
+      <x:c r="E58" s="6" t="n">
         <x:v>0.01879907644617325</x:v>
       </x:c>
-      <x:c r="F58" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G58" s="3" t="n">
+      <x:c r="F58" s="6" t="n">
         <x:v>0.003160914310062375</x:v>
       </x:c>
-      <x:c r="H58" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I58" s="3" t="n">
+      <x:c r="G58" s="6" t="n">
         <x:v>0.988929808139801</x:v>
       </x:c>
-      <x:c r="J58" s="3" t="n">
+      <x:c r="H58" s="6" t="n">
         <x:v>0.9961054921150208</x:v>
       </x:c>
-      <x:c r="K58" s="3" t="n">
+      <x:c r="I58" s="6" t="n">
         <x:v>0.9949561953544617</x:v>
       </x:c>
-      <x:c r="L58" s="3" t="n">
+      <x:c r="J58" s="6" t="n">
         <x:v>0.9964951872825623</x:v>
       </x:c>
-      <x:c r="M58" s="3" t="n">
+      <x:c r="K58" s="6" t="n">
         <x:v>0.9932920932769775</x:v>
       </x:c>
-      <x:c r="N58" s="3" t="n">
+      <x:c r="L58" s="6" t="n">
         <x:v>0.9930608868598938</x:v>
       </x:c>
+      <x:c r="M58" s="3"/>
+      <x:c r="N58" s="3"/>
     </x:row>
     <x:row r="59" ht="48">
       <x:c r="A59" s="3" t="str">
@@ -16499,36 +16301,32 @@
       <x:c r="D59" s="3" t="str">
         <x:v>ARHDEARPYFYRSSGYFDM</x:v>
       </x:c>
-      <x:c r="E59" s="3" t="n">
+      <x:c r="E59" s="6" t="n">
         <x:v>0.009530040486273325</x:v>
       </x:c>
-      <x:c r="F59" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G59" s="3" t="n">
+      <x:c r="F59" s="6" t="n">
         <x:v>0.02538070055650115</x:v>
       </x:c>
-      <x:c r="H59" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I59" s="3" t="n">
+      <x:c r="G59" s="6" t="n">
         <x:v>0.9790169596672058</x:v>
       </x:c>
-      <x:c r="J59" s="3" t="n">
+      <x:c r="H59" s="6" t="n">
         <x:v>0.9840048551559448</x:v>
       </x:c>
-      <x:c r="K59" s="3" t="n">
+      <x:c r="I59" s="6" t="n">
         <x:v>0.5096529722213745</x:v>
       </x:c>
-      <x:c r="L59" s="3" t="n">
+      <x:c r="J59" s="6" t="n">
         <x:v>0.9226171970367432</x:v>
       </x:c>
-      <x:c r="M59" s="3" t="n">
+      <x:c r="K59" s="6" t="n">
         <x:v>0.6939015984535217</x:v>
       </x:c>
-      <x:c r="N59" s="3" t="n">
+      <x:c r="L59" s="6" t="n">
         <x:v>0.986397922039032</x:v>
       </x:c>
+      <x:c r="M59" s="3"/>
+      <x:c r="N59" s="3"/>
     </x:row>
     <x:row r="60" ht="48">
       <x:c r="A60" s="3" t="str">
@@ -16543,36 +16341,32 @@
       <x:c r="D60" s="3" t="str">
         <x:v>ASGPHHSGSGTYYPSYLYG</x:v>
       </x:c>
-      <x:c r="E60" s="3" t="n">
+      <x:c r="E60" s="6" t="n">
         <x:v>0.03942976569368085</x:v>
       </x:c>
-      <x:c r="F60" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G60" s="3" t="n">
+      <x:c r="F60" s="6" t="n">
         <x:v>0.1112229472221345</x:v>
       </x:c>
-      <x:c r="H60" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I60" s="3" t="n">
+      <x:c r="G60" s="6" t="n">
         <x:v>0.0649641752243042</x:v>
       </x:c>
-      <x:c r="J60" s="3" t="n">
+      <x:c r="H60" s="6" t="n">
         <x:v>0.9915285110473633</x:v>
       </x:c>
-      <x:c r="K60" s="3" t="n">
+      <x:c r="I60" s="6" t="n">
         <x:v>0.02854940854012966</x:v>
       </x:c>
-      <x:c r="L60" s="3" t="n">
+      <x:c r="J60" s="6" t="n">
         <x:v>0.2691439688205719</x:v>
       </x:c>
-      <x:c r="M60" s="3" t="n">
+      <x:c r="K60" s="6" t="n">
         <x:v>0.007537475787103176</x:v>
       </x:c>
-      <x:c r="N60" s="3" t="n">
+      <x:c r="L60" s="6" t="n">
         <x:v>0.9601151943206787</x:v>
       </x:c>
+      <x:c r="M60" s="3"/>
+      <x:c r="N60" s="3"/>
     </x:row>
     <x:row r="61" ht="48">
       <x:c r="A61" s="3" t="str">
@@ -16587,36 +16381,32 @@
       <x:c r="D61" s="3" t="str">
         <x:v>ATRAIHFRNRNFYSFYVEV</x:v>
       </x:c>
-      <x:c r="E61" s="3" t="n">
+      <x:c r="E61" s="6" t="n">
         <x:v>0.3978048653319085</x:v>
       </x:c>
-      <x:c r="F61" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G61" s="3" t="n">
+      <x:c r="F61" s="6" t="n">
         <x:v>0.2356672891359393</x:v>
       </x:c>
-      <x:c r="H61" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I61" s="3" t="n">
+      <x:c r="G61" s="6" t="n">
         <x:v>0.001768490648828447</x:v>
       </x:c>
-      <x:c r="J61" s="3" t="n">
+      <x:c r="H61" s="6" t="n">
         <x:v>0.03476417064666748</x:v>
       </x:c>
-      <x:c r="K61" s="3" t="n">
+      <x:c r="I61" s="6" t="n">
         <x:v>0.005538433790206909</x:v>
       </x:c>
-      <x:c r="L61" s="3" t="n">
+      <x:c r="J61" s="6" t="n">
         <x:v>0.01239595655351877</x:v>
       </x:c>
-      <x:c r="M61" s="3" t="n">
+      <x:c r="K61" s="6" t="n">
         <x:v>0.001323652686551213</x:v>
       </x:c>
-      <x:c r="N61" s="3" t="n">
+      <x:c r="L61" s="6" t="n">
         <x:v>0.005618118215352297</x:v>
       </x:c>
+      <x:c r="M61" s="3"/>
+      <x:c r="N61" s="3"/>
     </x:row>
     <x:row r="62" ht="48">
       <x:c r="A62" s="3" t="str">
@@ -16631,36 +16421,32 @@
       <x:c r="D62" s="3" t="str">
         <x:v>AKDGRGLSIFGVLTPYYFDY</x:v>
       </x:c>
-      <x:c r="E62" s="3" t="n">
+      <x:c r="E62" s="6" t="n">
         <x:v>0.01038156111753612</x:v>
       </x:c>
-      <x:c r="F62" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G62" s="3" t="n">
+      <x:c r="F62" s="6" t="n">
         <x:v>0.04283239748829262</x:v>
       </x:c>
-      <x:c r="H62" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I62" s="3" t="n">
+      <x:c r="G62" s="6" t="n">
         <x:v>0.9512948989868164</x:v>
       </x:c>
-      <x:c r="J62" s="3" t="n">
+      <x:c r="H62" s="6" t="n">
         <x:v>0.9878726005554199</x:v>
       </x:c>
-      <x:c r="K62" s="3" t="n">
+      <x:c r="I62" s="6" t="n">
         <x:v>0.7425186634063721</x:v>
       </x:c>
-      <x:c r="L62" s="3" t="n">
+      <x:c r="J62" s="6" t="n">
         <x:v>0.9190903306007385</x:v>
       </x:c>
-      <x:c r="M62" s="3" t="n">
+      <x:c r="K62" s="6" t="n">
         <x:v>0.9715004563331604</x:v>
       </x:c>
-      <x:c r="N62" s="3" t="n">
+      <x:c r="L62" s="6" t="n">
         <x:v>0.9797878861427307</x:v>
       </x:c>
+      <x:c r="M62" s="3"/>
+      <x:c r="N62" s="3"/>
     </x:row>
     <x:row r="63" ht="48">
       <x:c r="A63" s="3" t="str">
@@ -16675,36 +16461,32 @@
       <x:c r="D63" s="3" t="str">
         <x:v>ARERVSMVRGIIMTYYGMDV</x:v>
       </x:c>
-      <x:c r="E63" s="3" t="n">
+      <x:c r="E63" s="6" t="n">
         <x:v>0.0450720918308392</x:v>
       </x:c>
-      <x:c r="F63" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G63" s="3" t="n">
+      <x:c r="F63" s="6" t="n">
         <x:v>0.04388350148511048</x:v>
       </x:c>
-      <x:c r="H63" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I63" s="3" t="n">
+      <x:c r="G63" s="6" t="n">
         <x:v>0.9310553073883057</x:v>
       </x:c>
-      <x:c r="J63" s="3" t="n">
+      <x:c r="H63" s="6" t="n">
         <x:v>0.5419207215309143</x:v>
       </x:c>
-      <x:c r="K63" s="3" t="n">
+      <x:c r="I63" s="6" t="n">
         <x:v>0.7965483665466309</x:v>
       </x:c>
-      <x:c r="L63" s="3" t="n">
+      <x:c r="J63" s="6" t="n">
         <x:v>0.8292937278747559</x:v>
       </x:c>
-      <x:c r="M63" s="3" t="n">
+      <x:c r="K63" s="6" t="n">
         <x:v>0.9512816667556763</x:v>
       </x:c>
-      <x:c r="N63" s="3" t="n">
+      <x:c r="L63" s="6" t="n">
         <x:v>0.945615291595459</x:v>
       </x:c>
+      <x:c r="M63" s="3"/>
+      <x:c r="N63" s="3"/>
     </x:row>
     <x:row r="64" ht="48">
       <x:c r="A64" s="3" t="str">
@@ -16719,36 +16501,32 @@
       <x:c r="D64" s="3" t="str">
         <x:v>ARGTITIFGPFIDRGYYFDY</x:v>
       </x:c>
-      <x:c r="E64" s="3" t="n">
+      <x:c r="E64" s="6" t="n">
         <x:v>0.0424681334512646</x:v>
       </x:c>
-      <x:c r="F64" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G64" s="3" t="n">
+      <x:c r="F64" s="6" t="n">
         <x:v>0.0732134685628746</x:v>
       </x:c>
-      <x:c r="H64" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I64" s="3" t="n">
+      <x:c r="G64" s="6" t="n">
         <x:v>0.934091329574585</x:v>
       </x:c>
-      <x:c r="J64" s="3" t="n">
+      <x:c r="H64" s="6" t="n">
         <x:v>0.9812907576560974</x:v>
       </x:c>
-      <x:c r="K64" s="3" t="n">
+      <x:c r="I64" s="6" t="n">
         <x:v>0.7826352119445801</x:v>
       </x:c>
-      <x:c r="L64" s="3" t="n">
+      <x:c r="J64" s="6" t="n">
         <x:v>0.8776922821998596</x:v>
       </x:c>
-      <x:c r="M64" s="3" t="n">
+      <x:c r="K64" s="6" t="n">
         <x:v>0.9385271072387695</x:v>
       </x:c>
-      <x:c r="N64" s="3" t="n">
+      <x:c r="L64" s="6" t="n">
         <x:v>0.9806326031684875</x:v>
       </x:c>
+      <x:c r="M64" s="3"/>
+      <x:c r="N64" s="3"/>
     </x:row>
     <x:row r="65" ht="48">
       <x:c r="A65" s="3" t="str">
@@ -16763,36 +16541,32 @@
       <x:c r="D65" s="3" t="str">
         <x:v>ARMGEWNLRLGDPYYHAMDV</x:v>
       </x:c>
-      <x:c r="E65" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F65" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G65" s="3" t="n">
+      <x:c r="E65" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F65" s="6" t="n">
         <x:v>0.09897801625686055</x:v>
       </x:c>
-      <x:c r="H65" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I65" s="3" t="n">
+      <x:c r="G65" s="6" t="n">
         <x:v>0.3149279356002808</x:v>
       </x:c>
-      <x:c r="J65" s="3" t="n">
+      <x:c r="H65" s="6" t="n">
         <x:v>0.35467728972435</x:v>
       </x:c>
-      <x:c r="K65" s="3" t="n">
+      <x:c r="I65" s="6" t="n">
         <x:v>0.3839203417301178</x:v>
       </x:c>
-      <x:c r="L65" s="3" t="n">
+      <x:c r="J65" s="6" t="n">
         <x:v>0.9342966675758362</x:v>
       </x:c>
-      <x:c r="M65" s="3" t="n">
+      <x:c r="K65" s="6" t="n">
         <x:v>0.02656432799994946</x:v>
       </x:c>
-      <x:c r="N65" s="3" t="n">
+      <x:c r="L65" s="6" t="n">
         <x:v>0.9032392501831055</x:v>
       </x:c>
+      <x:c r="M65" s="3"/>
+      <x:c r="N65" s="3"/>
     </x:row>
     <x:row r="66" ht="48">
       <x:c r="A66" s="3" t="str">
@@ -16807,36 +16581,32 @@
       <x:c r="D66" s="3" t="str">
         <x:v>ARVSEYDFWTGQRYYFYYMDV</x:v>
       </x:c>
-      <x:c r="E66" s="3" t="n">
+      <x:c r="E66" s="6" t="n">
         <x:v>0.00384859983162975</x:v>
       </x:c>
-      <x:c r="F66" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G66" s="3" t="n">
+      <x:c r="F66" s="6" t="n">
         <x:v>0.0497683678308503</x:v>
       </x:c>
-      <x:c r="H66" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I66" s="3" t="n">
+      <x:c r="G66" s="6" t="n">
         <x:v>0.9302641749382019</x:v>
       </x:c>
-      <x:c r="J66" s="3" t="n">
+      <x:c r="H66" s="6" t="n">
         <x:v>0.9293047189712524</x:v>
       </x:c>
-      <x:c r="K66" s="3" t="n">
+      <x:c r="I66" s="6" t="n">
         <x:v>0.9579781889915466</x:v>
       </x:c>
-      <x:c r="L66" s="3" t="n">
+      <x:c r="J66" s="6" t="n">
         <x:v>0.9969835877418518</x:v>
       </x:c>
-      <x:c r="M66" s="3" t="n">
+      <x:c r="K66" s="6" t="n">
         <x:v>0.7026221752166748</x:v>
       </x:c>
-      <x:c r="N66" s="3" t="n">
+      <x:c r="L66" s="6" t="n">
         <x:v>0.9932354092597961</x:v>
       </x:c>
+      <x:c r="M66" s="3"/>
+      <x:c r="N66" s="3"/>
     </x:row>
     <x:row r="67" ht="48">
       <x:c r="A67" s="3" t="str">
@@ -16851,36 +16621,32 @@
       <x:c r="D67" s="3" t="str">
         <x:v>ARLAEDYRSSSGFPRGYYFDY</x:v>
       </x:c>
-      <x:c r="E67" s="3" t="n">
+      <x:c r="E67" s="6" t="n">
         <x:v>0.232257530139242</x:v>
       </x:c>
-      <x:c r="F67" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G67" s="3" t="n">
+      <x:c r="F67" s="6" t="n">
         <x:v>0.204639460622062</x:v>
       </x:c>
-      <x:c r="H67" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I67" s="3" t="n">
+      <x:c r="G67" s="6" t="n">
         <x:v>0.0009895580587908626</x:v>
       </x:c>
-      <x:c r="J67" s="3" t="n">
+      <x:c r="H67" s="6" t="n">
         <x:v>0.9084368944168091</x:v>
       </x:c>
-      <x:c r="K67" s="3" t="n">
+      <x:c r="I67" s="6" t="n">
         <x:v>0.3267078399658203</x:v>
       </x:c>
-      <x:c r="L67" s="3" t="n">
+      <x:c r="J67" s="6" t="n">
         <x:v>0.5354183912277222</x:v>
       </x:c>
-      <x:c r="M67" s="3" t="n">
+      <x:c r="K67" s="6" t="n">
         <x:v>0.01492621470242739</x:v>
       </x:c>
-      <x:c r="N67" s="3" t="n">
+      <x:c r="L67" s="6" t="n">
         <x:v>0.9880808591842651</x:v>
       </x:c>
+      <x:c r="M67" s="3"/>
+      <x:c r="N67" s="3"/>
     </x:row>
     <x:row r="68" ht="48">
       <x:c r="A68" s="3" t="str">
@@ -16895,36 +16661,32 @@
       <x:c r="D68" s="3" t="str">
         <x:v>ARDDVGDGRNSDIHLRGDFEY</x:v>
       </x:c>
-      <x:c r="E68" s="3" t="n">
+      <x:c r="E68" s="6" t="n">
         <x:v>0.0272082696631216</x:v>
       </x:c>
-      <x:c r="F68" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G68" s="3" t="n">
+      <x:c r="F68" s="6" t="n">
         <x:v>0.0087441357177878</x:v>
       </x:c>
-      <x:c r="H68" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I68" s="3" t="n">
+      <x:c r="G68" s="6" t="n">
         <x:v>0.9893352389335632</x:v>
       </x:c>
-      <x:c r="J68" s="3" t="n">
+      <x:c r="H68" s="6" t="n">
         <x:v>0.9923117756843567</x:v>
       </x:c>
-      <x:c r="K68" s="3" t="n">
+      <x:c r="I68" s="6" t="n">
         <x:v>0.9911876916885376</x:v>
       </x:c>
-      <x:c r="L68" s="3" t="n">
+      <x:c r="J68" s="6" t="n">
         <x:v>0.991520345211029</x:v>
       </x:c>
-      <x:c r="M68" s="3" t="n">
+      <x:c r="K68" s="6" t="n">
         <x:v>0.9885397553443909</x:v>
       </x:c>
-      <x:c r="N68" s="3" t="n">
+      <x:c r="L68" s="6" t="n">
         <x:v>0.978492796421051</x:v>
       </x:c>
+      <x:c r="M68" s="3"/>
+      <x:c r="N68" s="3"/>
     </x:row>
     <x:row r="69" ht="48">
       <x:c r="A69" s="3" t="str">
@@ -16939,36 +16701,32 @@
       <x:c r="D69" s="3" t="str">
         <x:v>ARGLFGVLISKIRFSYYYMDV</x:v>
       </x:c>
-      <x:c r="E69" s="3" t="n">
+      <x:c r="E69" s="6" t="n">
         <x:v>0.03224407207278342</x:v>
       </x:c>
-      <x:c r="F69" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G69" s="3" t="n">
+      <x:c r="F69" s="6" t="n">
         <x:v>0.1008597450437528</x:v>
       </x:c>
-      <x:c r="H69" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I69" s="3" t="n">
+      <x:c r="G69" s="6" t="n">
         <x:v>0.2741317749023438</x:v>
       </x:c>
-      <x:c r="J69" s="3" t="n">
+      <x:c r="H69" s="6" t="n">
         <x:v>0.9804731011390686</x:v>
       </x:c>
-      <x:c r="K69" s="3" t="n">
+      <x:c r="I69" s="6" t="n">
         <x:v>0.4662456214427948</x:v>
       </x:c>
-      <x:c r="L69" s="3" t="n">
+      <x:c r="J69" s="6" t="n">
         <x:v>0.05833164229989052</x:v>
       </x:c>
-      <x:c r="M69" s="3" t="n">
+      <x:c r="K69" s="6" t="n">
         <x:v>0.1405458450317383</x:v>
       </x:c>
-      <x:c r="N69" s="3" t="n">
+      <x:c r="L69" s="6" t="n">
         <x:v>0.9481058120727539</x:v>
       </x:c>
+      <x:c r="M69" s="3"/>
+      <x:c r="N69" s="3"/>
     </x:row>
     <x:row r="70" ht="48">
       <x:c r="A70" s="3" t="str">
@@ -16983,36 +16741,32 @@
       <x:c r="D70" s="3" t="str">
         <x:v>ARLLEPTYYDILTGSNGYYFDY</x:v>
       </x:c>
-      <x:c r="E70" s="3" t="n">
+      <x:c r="E70" s="6" t="n">
         <x:v>0.01294509407636707</x:v>
       </x:c>
-      <x:c r="F70" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G70" s="3" t="n">
+      <x:c r="F70" s="6" t="n">
         <x:v>0.04991124272771255</x:v>
       </x:c>
-      <x:c r="H70" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I70" s="3" t="n">
+      <x:c r="G70" s="6" t="n">
         <x:v>0.6533681750297546</x:v>
       </x:c>
-      <x:c r="J70" s="3" t="n">
+      <x:c r="H70" s="6" t="n">
         <x:v>0.9928445219993591</x:v>
       </x:c>
-      <x:c r="K70" s="3" t="n">
+      <x:c r="I70" s="6" t="n">
         <x:v>0.9673234820365906</x:v>
       </x:c>
-      <x:c r="L70" s="3" t="n">
+      <x:c r="J70" s="6" t="n">
         <x:v>0.9974285960197449</x:v>
       </x:c>
-      <x:c r="M70" s="3" t="n">
+      <x:c r="K70" s="6" t="n">
         <x:v>0.05669355764985085</x:v>
       </x:c>
-      <x:c r="N70" s="3" t="n">
+      <x:c r="L70" s="6" t="n">
         <x:v>0.995776355266571</x:v>
       </x:c>
+      <x:c r="M70" s="3"/>
+      <x:c r="N70" s="3"/>
     </x:row>
     <x:row r="71" ht="48">
       <x:c r="A71" s="3" t="str">
@@ -17027,36 +16781,32 @@
       <x:c r="D71" s="3" t="str">
         <x:v>ARDQLTSTIVARALRYYPYMDV</x:v>
       </x:c>
-      <x:c r="E71" s="3" t="n">
+      <x:c r="E71" s="6" t="n">
         <x:v>0.3249519627018972</x:v>
       </x:c>
-      <x:c r="F71" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G71" s="3" t="n">
+      <x:c r="F71" s="6" t="n">
         <x:v>0.1603646064744125</x:v>
       </x:c>
-      <x:c r="H71" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I71" s="3" t="n">
+      <x:c r="G71" s="6" t="n">
         <x:v>0.04103982448577881</x:v>
       </x:c>
-      <x:c r="J71" s="3" t="n">
+      <x:c r="H71" s="6" t="n">
         <x:v>0.9796725511550903</x:v>
       </x:c>
-      <x:c r="K71" s="3" t="n">
+      <x:c r="I71" s="6" t="n">
         <x:v>0.9735852479934692</x:v>
       </x:c>
-      <x:c r="L71" s="3" t="n">
+      <x:c r="J71" s="6" t="n">
         <x:v>0.9323731660842896</x:v>
       </x:c>
-      <x:c r="M71" s="3" t="n">
+      <x:c r="K71" s="6" t="n">
         <x:v>0.912057638168335</x:v>
       </x:c>
-      <x:c r="N71" s="3" t="n">
+      <x:c r="L71" s="6" t="n">
         <x:v>0.9777725338935852</x:v>
       </x:c>
+      <x:c r="M71" s="3"/>
+      <x:c r="N71" s="3"/>
     </x:row>
     <x:row r="72" ht="48">
       <x:c r="A72" s="3" t="str">
@@ -17071,36 +16821,32 @@
       <x:c r="D72" s="3" t="str">
         <x:v>ARDRGLAGHYYDSNVYYGAFDI</x:v>
       </x:c>
-      <x:c r="E72" s="3" t="n">
+      <x:c r="E72" s="6" t="n">
         <x:v>0.001693450998483125</x:v>
       </x:c>
-      <x:c r="F72" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G72" s="3" t="n">
+      <x:c r="F72" s="6" t="n">
         <x:v>0.05351236438510218</x:v>
       </x:c>
-      <x:c r="H72" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I72" s="3" t="n">
+      <x:c r="G72" s="6" t="n">
         <x:v>0.957445502281189</x:v>
       </x:c>
-      <x:c r="J72" s="3" t="n">
+      <x:c r="H72" s="6" t="n">
         <x:v>0.8280432224273682</x:v>
       </x:c>
-      <x:c r="K72" s="3" t="n">
+      <x:c r="I72" s="6" t="n">
         <x:v>0.6624748706817627</x:v>
       </x:c>
-      <x:c r="L72" s="3" t="n">
+      <x:c r="J72" s="6" t="n">
         <x:v>0.7773358821868896</x:v>
       </x:c>
-      <x:c r="M72" s="3" t="n">
+      <x:c r="K72" s="6" t="n">
         <x:v>0.2957797944545746</x:v>
       </x:c>
-      <x:c r="N72" s="3" t="n">
+      <x:c r="L72" s="6" t="n">
         <x:v>0.9372302293777466</x:v>
       </x:c>
+      <x:c r="M72" s="3"/>
+      <x:c r="N72" s="3"/>
     </x:row>
     <x:row r="73" ht="48">
       <x:c r="A73" s="3" t="str">
@@ -17115,36 +16861,32 @@
       <x:c r="D73" s="3" t="str">
         <x:v>ARDNSFDPSDAVRDYYYYYMDV</x:v>
       </x:c>
-      <x:c r="E73" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F73" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G73" s="3" t="n">
+      <x:c r="E73" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F73" s="6" t="n">
         <x:v>0.01443521679746783</x:v>
       </x:c>
-      <x:c r="H73" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I73" s="3" t="n">
+      <x:c r="G73" s="6" t="n">
         <x:v>0.9927147030830383</x:v>
       </x:c>
-      <x:c r="J73" s="3" t="n">
+      <x:c r="H73" s="6" t="n">
         <x:v>0.9531859159469604</x:v>
       </x:c>
-      <x:c r="K73" s="3" t="n">
+      <x:c r="I73" s="6" t="n">
         <x:v>0.9891467094421387</x:v>
       </x:c>
-      <x:c r="L73" s="3" t="n">
+      <x:c r="J73" s="6" t="n">
         <x:v>0.9931069016456604</x:v>
       </x:c>
-      <x:c r="M73" s="3" t="n">
+      <x:c r="K73" s="6" t="n">
         <x:v>0.9921122789382935</x:v>
       </x:c>
-      <x:c r="N73" s="3" t="n">
+      <x:c r="L73" s="6" t="n">
         <x:v>0.9953598380088806</x:v>
       </x:c>
+      <x:c r="M73" s="3"/>
+      <x:c r="N73" s="3"/>
     </x:row>
     <x:row r="74" ht="48">
       <x:c r="A74" s="3" t="str">
@@ -17159,36 +16901,32 @@
       <x:c r="D74" s="3" t="str">
         <x:v>TRGVEDIVVVVAATPYYYYYMDV</x:v>
       </x:c>
-      <x:c r="E74" s="3" t="n">
+      <x:c r="E74" s="6" t="n">
         <x:v>0.009418580118484175</x:v>
       </x:c>
-      <x:c r="F74" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G74" s="3" t="n">
+      <x:c r="F74" s="6" t="n">
         <x:v>0.02478112040587945</x:v>
       </x:c>
-      <x:c r="H74" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I74" s="3" t="n">
+      <x:c r="G74" s="6" t="n">
         <x:v>0.9717898964881897</x:v>
       </x:c>
-      <x:c r="J74" s="3" t="n">
+      <x:c r="H74" s="6" t="n">
         <x:v>0.9969614148139954</x:v>
       </x:c>
-      <x:c r="K74" s="3" t="n">
+      <x:c r="I74" s="6" t="n">
         <x:v>0.9963453412055969</x:v>
       </x:c>
-      <x:c r="L74" s="3" t="n">
+      <x:c r="J74" s="6" t="n">
         <x:v>0.9917076230049133</x:v>
       </x:c>
-      <x:c r="M74" s="3" t="n">
+      <x:c r="K74" s="6" t="n">
         <x:v>0.9937006235122681</x:v>
       </x:c>
-      <x:c r="N74" s="3" t="n">
+      <x:c r="L74" s="6" t="n">
         <x:v>0.9944080114364624</x:v>
       </x:c>
+      <x:c r="M74" s="3"/>
+      <x:c r="N74" s="3"/>
     </x:row>
     <x:row r="75" ht="48">
       <x:c r="A75" s="3" t="str">
@@ -17203,36 +16941,32 @@
       <x:c r="D75" s="3" t="str">
         <x:v>ARDVGHFGDLLNFSAERSSLMDV</x:v>
       </x:c>
-      <x:c r="E75" s="3" t="n">
+      <x:c r="E75" s="6" t="n">
         <x:v>0.00462520476109295</x:v>
       </x:c>
-      <x:c r="F75" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G75" s="3" t="n">
+      <x:c r="F75" s="6" t="n">
         <x:v>0.03049250475917437</x:v>
       </x:c>
-      <x:c r="H75" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I75" s="3" t="n">
+      <x:c r="G75" s="6" t="n">
         <x:v>0.8635676503181458</x:v>
       </x:c>
-      <x:c r="J75" s="3" t="n">
+      <x:c r="H75" s="6" t="n">
         <x:v>0.9962748289108276</x:v>
       </x:c>
-      <x:c r="K75" s="3" t="n">
+      <x:c r="I75" s="6" t="n">
         <x:v>0.9389482736587524</x:v>
       </x:c>
-      <x:c r="L75" s="3" t="n">
+      <x:c r="J75" s="6" t="n">
         <x:v>0.9312453866004944</x:v>
       </x:c>
-      <x:c r="M75" s="3" t="n">
+      <x:c r="K75" s="6" t="n">
         <x:v>0.1059680208563805</x:v>
       </x:c>
-      <x:c r="N75" s="3" t="n">
+      <x:c r="L75" s="6" t="n">
         <x:v>0.9877421855926514</x:v>
       </x:c>
+      <x:c r="M75" s="3"/>
+      <x:c r="N75" s="3"/>
     </x:row>
     <x:row r="76" ht="48">
       <x:c r="A76" s="3" t="str">
@@ -17247,36 +16981,32 @@
       <x:c r="D76" s="3" t="str">
         <x:v>ARGGIQITVTTSLRPAYFYYMDV</x:v>
       </x:c>
-      <x:c r="E76" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F76" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G76" s="3" t="n">
+      <x:c r="E76" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F76" s="6" t="n">
         <x:v>0.09095060038616243</x:v>
       </x:c>
-      <x:c r="H76" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I76" s="3" t="n">
+      <x:c r="G76" s="6" t="n">
         <x:v>0.02870951406657696</x:v>
       </x:c>
-      <x:c r="J76" s="3" t="n">
+      <x:c r="H76" s="6" t="n">
         <x:v>0.987247884273529</x:v>
       </x:c>
-      <x:c r="K76" s="3" t="n">
+      <x:c r="I76" s="6" t="n">
         <x:v>0.9735191464424133</x:v>
       </x:c>
-      <x:c r="L76" s="3" t="n">
+      <x:c r="J76" s="6" t="n">
         <x:v>0.9534434676170349</x:v>
       </x:c>
-      <x:c r="M76" s="3" t="n">
+      <x:c r="K76" s="6" t="n">
         <x:v>0.8371973037719727</x:v>
       </x:c>
-      <x:c r="N76" s="3" t="n">
+      <x:c r="L76" s="6" t="n">
         <x:v>0.8816860318183899</x:v>
       </x:c>
+      <x:c r="M76" s="3"/>
+      <x:c r="N76" s="3"/>
     </x:row>
     <x:row r="77" ht="48">
       <x:c r="A77" s="3" t="str">
@@ -17291,36 +17021,32 @@
       <x:c r="D77" s="3" t="str">
         <x:v>ARGGIEGEILWWRDAGSDDAFDI</x:v>
       </x:c>
-      <x:c r="E77" s="3" t="n">
+      <x:c r="E77" s="6" t="n">
         <x:v>0.1019839606681215</x:v>
       </x:c>
-      <x:c r="F77" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G77" s="3" t="n">
+      <x:c r="F77" s="6" t="n">
         <x:v>0.04924106173348355</x:v>
       </x:c>
-      <x:c r="H77" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I77" s="3" t="n">
+      <x:c r="G77" s="6" t="n">
         <x:v>0.9765381217002869</x:v>
       </x:c>
-      <x:c r="J77" s="3" t="n">
+      <x:c r="H77" s="6" t="n">
         <x:v>0.9976173043251038</x:v>
       </x:c>
-      <x:c r="K77" s="3" t="n">
+      <x:c r="I77" s="6" t="n">
         <x:v>0.9982800483703613</x:v>
       </x:c>
-      <x:c r="L77" s="3" t="n">
+      <x:c r="J77" s="6" t="n">
         <x:v>0.9975893497467041</x:v>
       </x:c>
-      <x:c r="M77" s="3" t="n">
+      <x:c r="K77" s="6" t="n">
         <x:v>0.9931581616401672</x:v>
       </x:c>
-      <x:c r="N77" s="3" t="n">
+      <x:c r="L77" s="6" t="n">
         <x:v>0.9965470433235168</x:v>
       </x:c>
+      <x:c r="M77" s="3"/>
+      <x:c r="N77" s="3"/>
     </x:row>
     <x:row r="78" ht="64">
       <x:c r="A78" s="3" t="str">
@@ -17335,36 +17061,32 @@
       <x:c r="D78" s="3" t="str">
         <x:v>ARDSPPMGLGMGEYFGAYYYGMDV</x:v>
       </x:c>
-      <x:c r="E78" s="3" t="n">
+      <x:c r="E78" s="6" t="n">
         <x:v>0.2945326928609328</x:v>
       </x:c>
-      <x:c r="F78" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G78" s="3" t="n">
+      <x:c r="F78" s="6" t="n">
         <x:v>0.2025812974679218</x:v>
       </x:c>
-      <x:c r="H78" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I78" s="3" t="n">
+      <x:c r="G78" s="6" t="n">
         <x:v>0.884087085723877</x:v>
       </x:c>
-      <x:c r="J78" s="3" t="n">
+      <x:c r="H78" s="6" t="n">
         <x:v>0.97724449634552</x:v>
       </x:c>
-      <x:c r="K78" s="3" t="n">
+      <x:c r="I78" s="6" t="n">
         <x:v>0.9528493881225586</x:v>
       </x:c>
-      <x:c r="L78" s="3" t="n">
+      <x:c r="J78" s="6" t="n">
         <x:v>0.09620577096939087</x:v>
       </x:c>
-      <x:c r="M78" s="3" t="n">
+      <x:c r="K78" s="6" t="n">
         <x:v>0.006556234322488308</x:v>
       </x:c>
-      <x:c r="N78" s="3" t="n">
+      <x:c r="L78" s="6" t="n">
         <x:v>0.8142312169075012</x:v>
       </x:c>
+      <x:c r="M78" s="3"/>
+      <x:c r="N78" s="3"/>
     </x:row>
     <x:row r="79" ht="48">
       <x:c r="A79" s="3" t="str">
@@ -17379,36 +17101,32 @@
       <x:c r="D79" s="3" t="str">
         <x:v>ARASYDFWSGYYEPKKSATYAFDY</x:v>
       </x:c>
-      <x:c r="E79" s="3" t="n">
+      <x:c r="E79" s="6" t="n">
         <x:v>0.2692219762637993</x:v>
       </x:c>
-      <x:c r="F79" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G79" s="3" t="n">
+      <x:c r="F79" s="6" t="n">
         <x:v>0.1697741312988678</x:v>
       </x:c>
-      <x:c r="H79" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I79" s="3" t="n">
+      <x:c r="G79" s="6" t="n">
         <x:v>0.001067667850293219</x:v>
       </x:c>
-      <x:c r="J79" s="3" t="n">
+      <x:c r="H79" s="6" t="n">
         <x:v>0.0822225883603096</x:v>
       </x:c>
-      <x:c r="K79" s="3" t="n">
+      <x:c r="I79" s="6" t="n">
         <x:v>0.002123184502124786</x:v>
       </x:c>
-      <x:c r="L79" s="3" t="n">
+      <x:c r="J79" s="6" t="n">
         <x:v>0.001615225337445736</x:v>
       </x:c>
-      <x:c r="M79" s="3" t="n">
+      <x:c r="K79" s="6" t="n">
         <x:v>0.001225757761858404</x:v>
       </x:c>
-      <x:c r="N79" s="3" t="n">
+      <x:c r="L79" s="6" t="n">
         <x:v>0.9531373977661133</x:v>
       </x:c>
+      <x:c r="M79" s="3"/>
+      <x:c r="N79" s="3"/>
     </x:row>
     <x:row r="80" ht="48">
       <x:c r="A80" s="3" t="str">
@@ -17423,36 +17141,32 @@
       <x:c r="D80" s="3" t="str">
         <x:v>AHRVYYSDRSSYPRRPRIPSAFDY</x:v>
       </x:c>
-      <x:c r="E80" s="3" t="n">
+      <x:c r="E80" s="6" t="n">
         <x:v>0.4324273452395275</x:v>
       </x:c>
-      <x:c r="F80" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G80" s="3" t="n">
+      <x:c r="F80" s="6" t="n">
         <x:v>0.4170671585044612</x:v>
       </x:c>
-      <x:c r="H80" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I80" s="3" t="n">
+      <x:c r="G80" s="6" t="n">
         <x:v>0.6153112053871155</x:v>
       </x:c>
-      <x:c r="J80" s="3" t="n">
+      <x:c r="H80" s="6" t="n">
         <x:v>0.9489232897758484</x:v>
       </x:c>
-      <x:c r="K80" s="3" t="n">
+      <x:c r="I80" s="6" t="n">
         <x:v>0.1045529693365097</x:v>
       </x:c>
-      <x:c r="L80" s="3" t="n">
+      <x:c r="J80" s="6" t="n">
         <x:v>0.1806748360395432</x:v>
       </x:c>
-      <x:c r="M80" s="3" t="n">
+      <x:c r="K80" s="6" t="n">
         <x:v>0.001904281321913004</x:v>
       </x:c>
-      <x:c r="N80" s="3" t="n">
+      <x:c r="L80" s="6" t="n">
         <x:v>0.1277438700199127</x:v>
       </x:c>
+      <x:c r="M80" s="3"/>
+      <x:c r="N80" s="3"/>
     </x:row>
     <x:row r="81" ht="48">
       <x:c r="A81" s="3" t="str">
@@ -17467,36 +17181,32 @@
       <x:c r="D81" s="3" t="str">
         <x:v>AREGGSYYDILTGYYNGPPNWFDP</x:v>
       </x:c>
-      <x:c r="E81" s="3" t="n">
+      <x:c r="E81" s="6" t="n">
         <x:v>0.005848161303349825</x:v>
       </x:c>
-      <x:c r="F81" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G81" s="3" t="n">
+      <x:c r="F81" s="6" t="n">
         <x:v>0.01519038699562143</x:v>
       </x:c>
-      <x:c r="H81" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I81" s="3" t="n">
+      <x:c r="G81" s="6" t="n">
         <x:v>0.9558219909667969</x:v>
       </x:c>
-      <x:c r="J81" s="3" t="n">
+      <x:c r="H81" s="6" t="n">
         <x:v>0.9904318451881409</x:v>
       </x:c>
-      <x:c r="K81" s="3" t="n">
+      <x:c r="I81" s="6" t="n">
         <x:v>0.9773460626602173</x:v>
       </x:c>
-      <x:c r="L81" s="3" t="n">
+      <x:c r="J81" s="6" t="n">
         <x:v>0.9334639310836792</x:v>
       </x:c>
-      <x:c r="M81" s="3" t="n">
+      <x:c r="K81" s="6" t="n">
         <x:v>0.9663658142089844</x:v>
       </x:c>
-      <x:c r="N81" s="3" t="n">
+      <x:c r="L81" s="6" t="n">
         <x:v>0.990172266960144</x:v>
       </x:c>
+      <x:c r="M81" s="3"/>
+      <x:c r="N81" s="3"/>
     </x:row>
     <x:row r="82" ht="32">
       <x:c r="D82" s="3"/>

</xml_diff>